<commit_message>
small debug of max rows in historical kpi results
small debug of max rows in historical kpi results
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="545" documentId="8_{B8338304-AABB-44AF-8121-230B6192A46B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2F46657-34DB-4DEC-97DE-4F8FA1D8550C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A912466-C5BB-4C7E-A1D2-5E5E5DC5A2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t>Error Handling: If there are issues with your input (e.g., invalid dates, KPI Name not found), the scripts will provide error messages directly in the relevant cells or in a Log worksheet.</t>
-  </si>
-  <si>
-    <t>ETT_+0_on_test_kpi(1)</t>
   </si>
   <si>
     <r>
@@ -260,19 +257,22 @@
     <t xml:space="preserve">&lt; your apiKey </t>
   </si>
   <si>
-    <t>2025-03-28T06:59:00Z</t>
-  </si>
-  <si>
-    <t>2025-03-28T08:59:00Z</t>
-  </si>
-  <si>
-    <t>type your apiKey</t>
-  </si>
-  <si>
     <t>fromTime (ISO 8601 format)</t>
   </si>
   <si>
     <t>toTime (ISO 8601 format)</t>
+  </si>
+  <si>
+    <t>2025-03-29T00:01:00Z</t>
+  </si>
+  <si>
+    <t>2025-03-29T01:01:00Z</t>
+  </si>
+  <si>
+    <t>type api key here</t>
+  </si>
+  <si>
+    <t>kpi name here</t>
   </si>
 </sst>
 </file>
@@ -2606,7 +2606,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}" name="RequestLog" displayName="RequestLog" ref="A1:C2" insertRow="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}" name="RequestLog" displayName="RequestLog" ref="A1:C2" totalsRowShown="0">
   <autoFilter ref="A1:C2" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{4CDB99BC-04BC-4765-B14D-E8023F5CCD93}" name="Datetime"/>
@@ -2900,7 +2900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -2917,13 +2917,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -2931,10 +2931,10 @@
         <v>10</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>0</v>
@@ -2942,24 +2942,24 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>1</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
@@ -2967,7 +2967,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
         <v>6</v>
@@ -3011,17 +3011,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" s="1"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" s="1"/>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="1"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3040,7 +3043,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -3050,7 +3053,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -3085,42 +3088,42 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
@@ -3167,7 +3170,7 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3184,13 +3187,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3199,7 +3214,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -3428,7 +3443,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
@@ -3440,18 +3455,24 @@
 </scriptIds>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3459,7 +3480,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3478,28 +3499,11 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
     <ds:schemaRef ds:uri=""/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
now we have full calcualtion of travel times in historical kpis
now we have full calcualtion of travel times in historical kpis
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A912466-C5BB-4C7E-A1D2-5E5E5DC5A2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2595" documentId="8_{3A912466-C5BB-4C7E-A1D2-5E5E5DC5A2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54DA0BB0-10DE-4E53-9CA8-A97CC4E3698E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
   <si>
     <t>timeAggregation</t>
   </si>
@@ -263,16 +263,22 @@
     <t>toTime (ISO 8601 format)</t>
   </si>
   <si>
-    <t>2025-03-29T00:01:00Z</t>
-  </si>
-  <si>
-    <t>2025-03-29T01:01:00Z</t>
-  </si>
-  <si>
     <t>type api key here</t>
   </si>
   <si>
     <t>kpi name here</t>
+  </si>
+  <si>
+    <t>Body (answer)</t>
+  </si>
+  <si>
+    <t>Length (km)</t>
+  </si>
+  <si>
+    <t>2025-03-20T00:00:00Z</t>
+  </si>
+  <si>
+    <t>2025-03-20T10:00:00Z</t>
   </si>
 </sst>
 </file>
@@ -2588,30 +2594,28 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:D21" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A20:D21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:E21" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A20:E21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID"/>
     <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name"/>
     <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name"/>
     <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID"/>
+    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Length (km)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}" name="RequestLog" displayName="RequestLog" ref="A1:C2" totalsRowShown="0">
-  <autoFilter ref="A1:C2" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}" name="RequestLog" displayName="RequestLog" ref="A1:D3" totalsRowShown="0">
+  <autoFilter ref="A1:D3" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{4CDB99BC-04BC-4765-B14D-E8023F5CCD93}" name="Datetime"/>
     <tableColumn id="2" xr3:uid="{8772A88C-88FF-4465-A952-FF8C297A2798}" name="Request URL"/>
     <tableColumn id="3" xr3:uid="{B944E935-3BD2-4332-AD04-AB633DB393B2}" name="Status"/>
+    <tableColumn id="4" xr3:uid="{1DA005DA-F3ED-4515-9F91-5435A3F128C8}" name="Body (answer)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2900,14 +2904,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.7109375" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
-    <col min="5" max="5" width="117.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -2915,18 +2919,21 @@
     <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="K1" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -2940,24 +2947,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="K3" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -2965,7 +2975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>34</v>
       </c>
@@ -2973,31 +2983,31 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" s="2"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -3010,9 +3020,36 @@
       <c r="D20" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
@@ -3020,11 +3057,14 @@
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" s="1"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" s="1"/>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="1"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="1"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3167,14 +3207,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -3183,6 +3223,9 @@
       </c>
       <c r="C1" t="s">
         <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -3195,26 +3238,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -3443,6 +3466,26 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
@@ -3456,31 +3499,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3499,6 +3517,31 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
added TTI.BTI and BT
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luca.paone\github\PTV-Flows-tutorials\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D84D031-96B5-4282-BD41-83120E10E9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6A746C0-D85D-4AF5-A95F-06752455141A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
-    <sheet name="readme" sheetId="30" r:id="rId2"/>
-    <sheet name="Log" sheetId="95" r:id="rId3"/>
+    <sheet name="Log" sheetId="95" r:id="rId2"/>
+    <sheet name="README" sheetId="166" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -269,16 +269,16 @@
     <t>Length (km)</t>
   </si>
   <si>
-    <t>2025-03-20T10:00:00Z</t>
-  </si>
-  <si>
-    <t>2025-03-20T09:00:00Z</t>
-  </si>
-  <si>
-    <t>put your API key here</t>
-  </si>
-  <si>
     <t>kpi name</t>
+  </si>
+  <si>
+    <t>2025-03-01T09:00:00Z</t>
+  </si>
+  <si>
+    <t>2025-03-02T09:00:00Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> your apiKey </t>
   </si>
 </sst>
 </file>
@@ -471,14 +471,45 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -495,16 +526,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>466725</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1638300</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>82550</xdr:rowOff>
+      <xdr:rowOff>92075</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -522,7 +553,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2962275" y="3505200"/>
+          <a:off x="342900" y="3524250"/>
           <a:ext cx="1295400" cy="615950"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -576,15 +607,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>542925</xdr:colOff>
+      <xdr:colOff>590550</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1914525</xdr:colOff>
+      <xdr:colOff>1962150</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -602,7 +633,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="542925" y="1790700"/>
+          <a:off x="590550" y="1743075"/>
           <a:ext cx="1371600" cy="292100"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -657,97 +688,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>161924</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>400050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2000249</xdr:colOff>
+      <xdr:colOff>2105025</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>130175</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Rectangle: Rounded Corners 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{733F1F15-B2B6-4814-9154-9E704AD3B455}"/>
-            </a:ext>
-            <a:ext uri="{6ECC49D1-AA05-4338-93AA-15A1B29DFB0A}">
-              <asl:scriptLink xmlns:asl="http://schemas.microsoft.com/office/drawing/2021/scriptlink" val="{&quot;shareId&quot;:&quot;ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE&quot;}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2657474" y="2733675"/>
-          <a:ext cx="1838325" cy="292100"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="accent4">
-            <a:lumMod val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="accent1">
-              <a:shade val="15000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US"/>
-            <a:t>Get HDA KPI DETAILED data</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-150"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2352675</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>180974</xdr:rowOff>
+      <xdr:rowOff>66674</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -765,7 +714,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="257175" y="2705100"/>
+          <a:off x="2505075" y="2600325"/>
           <a:ext cx="2095500" cy="371474"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -825,15 +774,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123824</xdr:colOff>
+      <xdr:colOff>2324099</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2495549</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2200274</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>149225</xdr:rowOff>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -851,7 +800,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="123824" y="3705225"/>
+          <a:off x="2324099" y="3724275"/>
           <a:ext cx="2371725" cy="292100"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -894,7 +843,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="it-IT"/>
-            <a:t>Get KPI Percentiles and  Pivot data</a:t>
+            <a:t>Get KPI Percentiles and  Indexes</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -906,13 +855,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1949450</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -930,7 +879,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2705100" y="1790700"/>
+          <a:off x="2705100" y="1743075"/>
           <a:ext cx="1739900" cy="292100"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -986,15 +935,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>409575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1047751</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1012,14 +961,16 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5400675" y="2743200"/>
-          <a:ext cx="2628900" cy="292100"/>
+          <a:off x="4838700" y="2609850"/>
+          <a:ext cx="2638426" cy="390525"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="107C41"/>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
         </a:solidFill>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
@@ -1065,15 +1016,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1914525</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:colOff>1962150</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1091,8 +1042,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1914525" y="1936750"/>
-          <a:ext cx="790575" cy="0"/>
+          <a:off x="1962150" y="1889125"/>
+          <a:ext cx="742950" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1122,14 +1073,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1949450</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
+      <xdr:colOff>123825</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:rowOff>90488</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1147,8 +1098,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4445000" y="1936750"/>
-          <a:ext cx="955675" cy="952500"/>
+          <a:off x="4445000" y="1889125"/>
+          <a:ext cx="393700" cy="915988"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -1179,15 +1130,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1228725</xdr:colOff>
+      <xdr:colOff>1276349</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1304925</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1057274</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>400050</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1205,8 +1156,66 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm rot="16200000" flipH="1">
-          <a:off x="955675" y="2355850"/>
-          <a:ext cx="622300" cy="76200"/>
+          <a:off x="2132012" y="1179512"/>
+          <a:ext cx="565150" cy="2276475"/>
+        </a:xfrm>
+        <a:prstGeom prst="curvedConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1014412</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1057275</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>57151</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="8" name="Connector: Curved 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{796D5127-520E-4B27-96F4-9028B9B021A8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="2" idx="2"/>
+          <a:endCxn id="5" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="3155156" y="3326606"/>
+          <a:ext cx="752476" cy="42863"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -1237,131 +1246,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1228726</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>177799</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1081088</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>28574</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="19" name="Connector: Curved 18">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C923D7B5-381D-4F31-9F05-5B51CB983333}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="4" idx="2"/>
-          <a:endCxn id="6" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="16200000" flipH="1">
-          <a:off x="2077244" y="1234281"/>
-          <a:ext cx="650875" cy="2347912"/>
-        </a:xfrm>
-        <a:prstGeom prst="curvedConnector3">
-          <a:avLst>
-            <a:gd name="adj1" fmla="val 50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1304926</xdr:colOff>
+      <xdr:colOff>990601</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>180973</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1309688</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>47624</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="8" name="Connector: Curved 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{796D5127-520E-4B27-96F4-9028B9B021A8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="2" idx="2"/>
-          <a:endCxn id="5" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="16200000" flipH="1">
-          <a:off x="992981" y="3398043"/>
-          <a:ext cx="628651" cy="4762"/>
-        </a:xfrm>
-        <a:prstGeom prst="curvedConnector3">
-          <a:avLst>
-            <a:gd name="adj1" fmla="val 50000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1081088</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>130174</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1114426</xdr:colOff>
+      <xdr:colOff>1304926</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>38099</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1373,14 +1266,15 @@
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="6" idx="2"/>
+          <a:cxnSpLocks/>
+          <a:stCxn id="51" idx="2"/>
           <a:endCxn id="3" idx="0"/>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm rot="16200000" flipH="1">
-          <a:off x="3353594" y="3248818"/>
-          <a:ext cx="479425" cy="33338"/>
+        <a:xfrm rot="5400000">
+          <a:off x="876301" y="3095625"/>
+          <a:ext cx="542925" cy="314325"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -1411,9 +1305,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>38099</xdr:rowOff>
+      <xdr:colOff>990600</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47624</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1429,7 +1323,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="123825" y="1752599"/>
+          <a:off x="990600" y="1390649"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -1580,9 +1474,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>800100</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>104774</xdr:rowOff>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>276224</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1598,7 +1492,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="800100" y="2305049"/>
+          <a:off x="228600" y="2190749"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -1749,9 +1643,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2028825</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>47624</xdr:rowOff>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123824</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1767,7 +1661,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4524375" y="1571624"/>
+          <a:off x="2505075" y="1276349"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -1918,9 +1812,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>695325</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>247650</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1936,7 +1830,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5410200" y="3086100"/>
+          <a:off x="4829175" y="2162175"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -2087,9 +1981,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:colOff>1133475</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
+      <xdr:rowOff>28574</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -2105,7 +1999,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3686175" y="2333624"/>
+          <a:off x="3629025" y="2228849"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -2255,18 +2149,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1819275</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1314450</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="TextBox 25">
+        <xdr:cNvPr id="27" name="TextBox 26">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45FB32C4-B8DC-4ECD-82CC-022FEC12A974}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3F141A5-08C5-4478-A96E-18202DB7FB09}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2274,7 +2168,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4314825" y="3514725"/>
+          <a:off x="1314450" y="3133725"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -2424,18 +2318,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>876300</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="TextBox 26">
+        <xdr:cNvPr id="28" name="TextBox 27">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3F141A5-08C5-4478-A96E-18202DB7FB09}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D61170A-6A11-4845-AECF-4531FAF1098B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2443,7 +2337,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="876300" y="3305175"/>
+          <a:off x="2952750" y="3305175"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -2591,6 +2485,224 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>400050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2352675</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="Rectangle: Rounded Corners 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C678E822-8471-48B2-A8A7-E1A5025ADC87}"/>
+            </a:ext>
+            <a:ext uri="{6ECC49D1-AA05-4338-93AA-15A1B29DFB0A}">
+              <asl:scriptLink xmlns:asl="http://schemas.microsoft.com/office/drawing/2021/scriptlink" val="{&quot;shareId&quot;:&quot;ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE&quot;}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="257175" y="2600325"/>
+          <a:ext cx="2095500" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="it-IT"/>
+            <a:t>Get KPI DETAILED results</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1276349</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1304924</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>400050</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="52" name="Connector: Curved 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A533DAE-0F96-4F43-BE83-0E1A4CDE0F8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="4" idx="2"/>
+          <a:endCxn id="51" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000" flipH="1">
+          <a:off x="1008062" y="2303462"/>
+          <a:ext cx="565150" cy="28575"/>
+        </a:xfrm>
+        <a:prstGeom prst="curvedConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>771524</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>171449</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="Rectangle: Rounded Corners 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48A913AB-B34C-47A3-90BC-5A9C43F28400}"/>
+            </a:ext>
+            <a:ext uri="{6ECC49D1-AA05-4338-93AA-15A1B29DFB0A}">
+              <asl:scriptLink xmlns:asl="http://schemas.microsoft.com/office/drawing/2021/scriptlink" val="{&quot;shareId&quot;:&quot;ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE&quot;}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9715499" y="1724025"/>
+          <a:ext cx="1628775" cy="666750"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="it-IT"/>
+            <a:t>Delete Temporary KPI tabs and clean logs</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2609,13 +2721,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}" name="RequestLog" displayName="RequestLog" ref="A1:D9" totalsRowShown="0">
-  <autoFilter ref="A1:D9" xr:uid="{471C674A-C50B-4F66-B9E0-64C2FEA1DBB0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="57" xr:uid="{4779B11E-4C20-4CE8-AC37-1278C30D0133}" name="RequestLog" displayName="RequestLog" ref="A1:D2" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:D2" xr:uid="{4779B11E-4C20-4CE8-AC37-1278C30D0133}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4CDB99BC-04BC-4765-B14D-E8023F5CCD93}" name="Datetime"/>
-    <tableColumn id="2" xr3:uid="{8772A88C-88FF-4465-A952-FF8C297A2798}" name="Request URL"/>
-    <tableColumn id="3" xr3:uid="{B944E935-3BD2-4332-AD04-AB633DB393B2}" name="Status"/>
-    <tableColumn id="4" xr3:uid="{1DA005DA-F3ED-4515-9F91-5435A3F128C8}" name="Body (answer)"/>
+    <tableColumn id="1" xr3:uid="{E4A4D8F0-6389-487C-B553-3695479C90CE}" name="Datetime" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{77E696F4-D736-472C-BCA0-1C09B9AD8961}" name="Request URL" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{E4DBE4B1-88AB-4591-A09B-D68B67461633}" name="Status" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{A104AB7D-241D-4758-8B3F-91AB794AA629}" name="Body (answer)" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2904,7 +3016,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K122"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -2924,7 +3036,7 @@
         <v>40</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>41</v>
@@ -2947,13 +3059,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>46</v>
+      <c r="C3" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>8</v>
@@ -3020,6 +3132,30 @@
         <v>45</v>
       </c>
     </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+    </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
     </row>
@@ -3047,8 +3183,8 @@
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
@@ -3074,20 +3210,50 @@
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
     </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1"/>
+    </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1"/>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" s="1"/>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" s="1"/>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" s="1"/>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="1"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="1"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="1"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" s="1"/>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3100,7 +3266,47 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD0D82FA-FD42-4D62-AAF4-10567937BF75}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A57C2C16-3654-4C73-B5DD-4EE8172FF9A3}">
   <dimension ref="A1:A37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3224,39 +3430,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -3490,15 +3663,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
@@ -3507,6 +3671,15 @@
     <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3518,6 +3691,7 @@
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
 </scriptIds>
 </file>
 
@@ -3541,14 +3715,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -3565,6 +3731,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
now dates and times are vaildated and protected by mistakes
now dates and times are vaildated and so protected by mistakes
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="798" documentId="13_ncr:1_{D9CF336E-4AE6-405D-A786-F5B1F48FC817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56AC15FD-BD8B-4535-8824-6C40C814F792}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95DDA57B-3676-45BB-A66F-CCDE6B669731}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,43 +37,82 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}</author>
+    <author>tc={B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Attention, Time and Date in UTC</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="1" shapeId="0" xr:uid="{B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Attention, Time and Date in UTC</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
-  <si>
-    <t>timeAggregation</t>
-  </si>
-  <si>
-    <t>MINUTES_5</t>
-  </si>
-  <si>
-    <t>KPI ID</t>
-  </si>
-  <si>
-    <t>KPI Name</t>
-  </si>
-  <si>
-    <t>Location Name</t>
-  </si>
-  <si>
-    <t>Location ID</t>
-  </si>
-  <si>
-    <t>MINUTES_15</t>
-  </si>
-  <si>
-    <t>MINUTES_30</t>
-  </si>
-  <si>
-    <t>HOURS_1</t>
-  </si>
-  <si>
-    <t>DAYS_1</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
+  <si>
+    <t>your apiKey &gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt; your apiKey </t>
   </si>
   <si>
     <t>KPI NAME
  (copy from the KPI table below)</t>
   </si>
   <si>
+    <t>timeAggregation</t>
+  </si>
+  <si>
+    <t>MINUTES_5</t>
+  </si>
+  <si>
+    <t>&lt;- copy and paste your choice for timeAggregation (MINUTES5,MINUTES15,etc)</t>
+  </si>
+  <si>
+    <t>Click on the buttons below and follow one of the possible workflows</t>
+  </si>
+  <si>
+    <t>MINUTES_15</t>
+  </si>
+  <si>
+    <t>MINUTES_30</t>
+  </si>
+  <si>
+    <t>HOURS_1</t>
+  </si>
+  <si>
+    <t>DAYS_1</t>
+  </si>
+  <si>
+    <t>KPI ID</t>
+  </si>
+  <si>
+    <t>KPI Name</t>
+  </si>
+  <si>
+    <t>Location Name</t>
+  </si>
+  <si>
+    <t>Location ID</t>
+  </si>
+  <si>
     <t>Datetime</t>
   </si>
   <si>
@@ -83,43 +122,13 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Body (answer)</t>
+  </si>
+  <si>
+    <t>README v 0.9</t>
+  </si>
+  <si>
     <t>Create an API key from your PTV Flows instance and copy it into the Config tab, cell B1.</t>
-  </si>
-  <si>
-    <t>Select the From and To dates in cells B3 and C3 respectively.</t>
-  </si>
-  <si>
-    <t>NOTE:</t>
-  </si>
-  <si>
-    <t>You can use the TomTom demo decoder at https://demo.tomtom.com/ to check the position of the OpenLR code.</t>
-  </si>
-  <si>
-    <t>Date Format: Dates must be in ISO 8601 format to be correctly processed by the scripts and API.</t>
-  </si>
-  <si>
-    <t>This will retrieve the list of available KPIs and populate the KPI_list table with their IDs, names, and associated locations.</t>
-  </si>
-  <si>
-    <t>In the Config tab, cell A3, enter the name of the KPI from which you want to get the data.</t>
-  </si>
-  <si>
-    <t>Ensure that the KPI name matches exactly as listed in the KPI_list table.</t>
-  </si>
-  <si>
-    <t>Dates should be in ISO 8601 format (e.g., 2023-01-01T00:00:00Z).</t>
-  </si>
-  <si>
-    <t>The From date must be before the To date.</t>
-  </si>
-  <si>
-    <t>Important Notes:</t>
-  </si>
-  <si>
-    <t>Time Aggregation (if applicable): Ensure that any time aggregation parameters are entered correctly in the appropriate cell (e.g., cell D3) with valid values like "MINUTES_5", "HOURS_1", etc.</t>
-  </si>
-  <si>
-    <t>Error Handling: If there are issues with your input (e.g., invalid dates, KPI Name not found), the scripts will provide error messages directly in the relevant cells or in a Log worksheet.</t>
   </si>
   <si>
     <r>
@@ -148,101 +157,25 @@
     </r>
   </si>
   <si>
+    <t>This will retrieve the list of available KPIs and populate the KPI_list table with their IDs, names, and associated locations.</t>
+  </si>
+  <si>
+    <t>In the Config tab, cell A3, enter the name of the KPI from which you want to get the data.</t>
+  </si>
+  <si>
+    <t>Ensure that the KPI name matches exactly as listed in the KPI_list table.</t>
+  </si>
+  <si>
+    <t>Select the From and To dates in cells B3 and C3 respectively.</t>
+  </si>
+  <si>
+    <t>Dates should be in ISO 8601 format (e.g., 2023-01-01T00:00:00Z).</t>
+  </si>
+  <si>
+    <t>The From date must be before the To date.</t>
+  </si>
+  <si>
     <t>For the "Get HDA KPI DETAILED data" button, the time interval between From and To should not exceed 24 hours.</t>
-  </si>
-  <si>
-    <t>&lt;- copy and paste your choice for timeAggregation (MINUTES5,MINUTES15,etc)</t>
-  </si>
-  <si>
-    <t>Click on the buttons below and follow one of the possible workflows</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">IN </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="5"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>orange</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : cells THAT CAN BE EDITED BY THE USER</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Once you have the Location you will be able to generate KPI overall results and detailed data  for a KPI also BEFORE it was created for the desired time range </t>
-  </si>
-  <si>
-    <t>your apiKey &gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt; your apiKey </t>
-  </si>
-  <si>
-    <t>fromTime (ISO 8601 format)</t>
-  </si>
-  <si>
-    <t>toTime (ISO 8601 format)</t>
-  </si>
-  <si>
-    <t>Body (answer)</t>
-  </si>
-  <si>
-    <t>Length (km)</t>
-  </si>
-  <si>
-    <t>README v 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PREREQUISITES </t>
-  </si>
-  <si>
-    <r>
-      <t>* Microsoft Excel *</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Desktop</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>* version</t>
-    </r>
-  </si>
-  <si>
-    <t>* PTV Flows API Key</t>
-  </si>
-  <si>
-    <t>* An Office 365 work or schoool account</t>
-  </si>
-  <si>
-    <t>GUIDE</t>
   </si>
   <si>
     <r>
@@ -257,7 +190,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Get overall Kpi results</t>
+      <t>Get HDA overall Kpi results</t>
     </r>
     <r>
       <rPr>
@@ -278,7 +211,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Get KPI DETAILED results</t>
+      <t>Get HDA KPI DETAILED data</t>
     </r>
     <r>
       <rPr>
@@ -292,47 +225,159 @@
     </r>
   </si>
   <si>
-    <t>Get overall Kpi results: Retrieves aggregated KPI data over the selected time range.</t>
-  </si>
-  <si>
-    <t>GetKPI DETAILED data: Retrieves detailed KPI data (including values for each road link of the KPI) within the selected time range.</t>
-  </si>
-  <si>
-    <t>Create KPI heatmap : Create the heatmap for the detailed results in the related tab</t>
-  </si>
-  <si>
-    <t>Get KPI Percentiles and  Indexes : create the percentiles and average and Indexes like TTI,BTI, for further analysis for the overall results. Various tabs will be created accordingly</t>
-  </si>
-  <si>
-    <t>After you have downloaded the KPI definitions and you have chosen a KPI you can also click on "Get KPI Locations Details" that will give you details on the Location of the KPI (road links, order, OpenLRcode) in the tab with the same name</t>
+    <t>Get HDA overall Kpi results: Retrieves aggregated KPI data over the selected time range.</t>
+  </si>
+  <si>
+    <t>Get HDA KPI DETAILED data: Retrieves detailed KPI data (including values for each road link of the KPI) within the selected time range.</t>
+  </si>
+  <si>
+    <t>Create the heatmap for the detailed results in the related tab</t>
+  </si>
+  <si>
+    <t>OR create the pivot data and percentiles for further analysis for the overall results. Various tabs will be created accordingly</t>
+  </si>
+  <si>
+    <t>After you have downloaded the KPI definitinos and oyu have chosen a KPI you can also click on "Get KPI Locations Details" that will give you details on the Location of the KPI (road links, order, OpenLRcode) in the tab with the same name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Once you have the Location you will be able to generate KPI overall results and detailed data  for a KPI also BEFORE it was created for the desired time range </t>
+  </si>
+  <si>
+    <t>NOTE:</t>
+  </si>
+  <si>
+    <t>You can use the TomTom demo decoder at https://demo.tomtom.com/ to check the position of the OpenLR code.</t>
+  </si>
+  <si>
+    <t>Important Notes:</t>
+  </si>
+  <si>
+    <t>Date Format: Dates must be in ISO 8601 format to be correctly processed by the scripts and API.</t>
+  </si>
+  <si>
+    <t>Time Aggregation (if applicable): Ensure that any time aggregation parameters are entered correctly in the appropriate cell (e.g., cell D3) with valid values like "MINUTES_5", "HOURS_1", etc.</t>
+  </si>
+  <si>
+    <t>Error Handling: If there are issues with your input (e.g., invalid dates, KPI Name not found), the scripts will provide error messages directly in the relevant cells or in a Log worksheet.</t>
+  </si>
+  <si>
+    <t>Note:to use the Script oyu need a work or home account</t>
   </si>
   <si>
     <t>Subscription id (in the PTV FLOWS URL)</t>
   </si>
   <si>
+    <t>Km Length</t>
+  </si>
+  <si>
     <t>KPI url</t>
   </si>
   <si>
-    <t>2025-03-07T23:59:00Z</t>
-  </si>
-  <si>
-    <t>2025-03-01T00:00:00Z</t>
-  </si>
-  <si>
-    <t>kpi NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">apiKey </t>
-  </si>
-  <si>
-    <t>your subscription id</t>
+    <t>https://api.ptvgroup.tech/kpieng/v1/instance/all</t>
+  </si>
+  <si>
+    <t>Success: Retrieved 17 KPIs</t>
+  </si>
+  <si>
+    <t>[{"name":"ETT_+20_on_FCO-Tuscolana","notes":"","kpiInstanceParameters":{"parameters":{"timetostart":1200}},"location":{"name":"FCO-Tuscolana","shape":"LINESTRING (12.268298 41.787941, 12.27342 41.79023, 12.28064 41.79425, 12.28259 41.79533, 12.28786 41.79827, 12.28902 41.7989, 12.29347 41.8014, 12.29597 41.80279, 12.29658 41.80313, 12.29929 41.80467, 12.29976 41.80493, 12.30317 41.80683, 12.30442 41.80752, 12.30472 41.80768, 12.30593 41.80832, 12.30652 41.80859, 12.31006 41.81001, 12.31084 41.81026, 12.3122 41.81065, 12.31543 41.81139, 12.31812 41.81177, 12.31881 41.81184, 12.31935 41.81189, 12.32066 41.812, 12.3218 41.81212, 12.32213 41.81214, 12.32279 41.81221, 12.32427 41.81233, 12.3244 41.81234, 12.32537 41.81243, 12.32683 41.81256, 12.32704 41.81258, 12.3335 41.81316, 12.3337 41.81317, 12.33761 41.81354, 12.33939 41.8137, 12.33952 41.81371, 12.34127 41.81386, 12.34254 41.81398, 12.34696 41.81437, 12.3471 41.81438, 12.34804 41.81447, 12.34895 41.81454, 12.35603 41.81518, 12.36148 41.81567, 12.36213 41.81572, 12.36498 41.81597, 12.36893 41.81632, 12.36941 41.81636, 12.37122 41.81654, 12.37245 41.81655, 12.37293 41.81658, 12.37544 41.81676, 12.37606 41.81682, 12.37629 41.81683, 12.37643 41.81684, 12.37671 41.81687, 12.37845 41.81703, 12.38538 41.81762, 12.38562 41.81764, 12.38774 41.81767, 12.38837 41.81758, 12.38956 41.81718, 12.39186 41.81608, 12.39233 41.81575, 12.3931 41.81508, 12.39347 41.81473, 12.3942 41.81411, 12.39585 41.81295, 12.39789 41.81182, 12.3983 41.81162, 12.39841 41.81158, 12.39901 41.81134, 12.40003 41.81096, 12.40153 41.81055, 12.40264 41.81034, 12.4052 41.80975, 12.40598 41.80957, 12.41072 41.80871, 12.4122 41.80849, 12.41494 41.80811, 12.41591 41.80798, 12.4176 41.80774, 12.41793 41.80768, 12.41841 41.80761, 12.41858 41.80759, 12.4194 41.80747, 12.4198 41.80742, 12.41999 41.80739, 12.42042 41.80732, 12.42077 41.80727, 12.42127 41.80718, 12.42248 41.80688, 12.42457 41.80624, 12.4326 41.80362, 12.43585 41.80298, 12.43625 41.80292, 12.43657 41.80288, 12.43668 41.80287, 12.4393 41.80257, 12.44016 41.80248, 12.4422 41.80223, 12.44434 41.80197, 12.44444 41.80196, 12.44478 41.80192, 12.44502 41.80189, 12.44572 41.8018, 12.446 41.80177, 12.44767 41.80156, 12.44829 41.80148, 12.44984 41.8013, 12.44993 41.80129, 12.45316 41.80087, 12.45358 41.80082, 12.45374 41.8008, 12.45395 41.80078, 12.45417 41.80075, 12.4566 41.80046, 12.45748 41.80034, 12.45831 41.80024, 12.4593 41.80012, 12.46124 41.79989, 12.46577 41.79934, 12.4714 41.79865, 12.47545 41.79816, 12.47559 41.79814, 12.47575 41.79812, 12.47604 41.7981, 12.47643 41.79805, 12.47708 41.79796, 12.48015 41.79759, 12.48065 41.79753, 12.48079 41.79752, 12.48097 41.79749, 12.48126 41.79746, 12.48422 41.7971, 12.48461 41.79705, 12.48558 41.79693, 12.49026 41.79636, 12.49957 41.79525, 12.50449 41.79465, 12.50705 41.79433, 12.50787 41.79425, 12.50835 41.79421, 12.51102 41.79412, 12.51118 41.79411, 12.5118 41.79413, 12.51355 41.79421, 12.51369 41.79422, 12.51413 41.79425, 12.51563 41.79437, 12.51616 41.79442, 12.52077 41.7948, 12.52142 41.79486, 12.52244 41.79495, 12.52544 41.79526, 12.52803 41.79572, 12.52858 41.79584, 12.53114 41.79639, 12.53235 41.79666, 12.53419 41.79705, 12.53463 41.79715, 12.5356 41.79737, 12.53748 41.79778, 12.5377 41.79783, 12.5379 41.79787, 12.53806 41.79791, 12.53902 41.79812, 12.53985 41.79831, 12.54864 41.8002, 12.55144 41.80098, 12.55159 41.80103, 12.55502 41.80238, 12.55681 41.80329, 12.55706 41.80343, 12.55773 41.80378, 12.55896 41.80449, 12.55981 41.80495, 12.56118 41.80573, 12.56325 41.80688, 12.56817 41.80966, 12.56936 41.81032, 12.56972 41.81054, 12.5701 41.81075, 12.57037 41.8109, 12.57284 41.81236, 12.57289 41.81239, 12.57299 41.81245, 12.57437 41.81359, 12.57527 41.81465, 12.57563 41.81515, 12.57589 41.81556, 12.57626 41.81612, 12.57707 41.81731, 12.57715 41.81744, 12.57732 41.8177, 12.57811 41.81888, 12.57861 41.81964, 12.57888 41.82002, 12.57903 41.82026, 12.57928 41.82045, 12.57974 41.82093, 12.57977 41.82097, 12.58047 41.82182, 12.5806 41.822, 12.58065 41.82208, 12.58078 41.82229, 12.58094 41.82256, 12.581 41.82266, 12.58108 41.82281, 12.58133 41.82327, 12.58156 41.82378, 12.58226 41.82484, 12.58254 41.82528, 12.58302 41.82598, 12.58359 41.82687, 12.5843 41.82807, 12.58439 41.82821, 12.58454 41.82845, 12.58486 41.82898, 12.58564 41.83015, 12.5864 41.83125, 12.58676 41.83182, 12.58716 41.83241, 12.58731 41.83262, 12.58764 41.83306, 12.5877 41.83314, 12.58782 41.83326, 12.58824 41.83352, 12.58844 41.83375, 12.58879 41.83416, 12.58903 41.83468, 12.58943 41.83523, 12.58991 41.83555, 12.59065 41.83603, 12.59136 41.83621, 12.59173 41.83609, 12.59244 41.83561, 12.59303 41.83505, 12.5933 41.83477, 12.59348 41.83461, 12.59384 41.83424)","locationId":"c9e15a7d-b590-4720-827e-303a5b387b08","locationType":"PATH"},"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","thresholdsDefinition":{"thresholdsValues":{"warningThreshold":90.0,"criticalThreshold":100.0},"kpiThresholdsReference":"UNUSUAL"},"template":"EXPECTED_TRAVEL_TIME"...</t>
+  </si>
+  <si>
+    <t>Error: {"message":"You cannot perform the requested operation.","code":"AccessDenied","type":"Table","method":"deleteRowsAt","line":223}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kpi name </t>
+  </si>
+  <si>
+    <t>2025-04-07T14:33:48.723Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:33:48.826Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:37:03.024Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:37:03.130Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:40:15.981Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:40:16.327Z</t>
+  </si>
+  <si>
+    <t>https://api.ptvgroup.tech/kpieng/v1/result/by-kpi-ids</t>
+  </si>
+  <si>
+    <t>Success: Retrieved length data for 34 KPIs</t>
+  </si>
+  <si>
+    <t>[{"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","timeStamp":"2025-04-07T14:32:00Z","results":[{"value":0.7160851,"defaultValue":0.67702585,"unusualValue":0.75992703,"averageValue":0.3549224,"progressive":1.2412142},{"value":0.113773584,"defaultValue":0.10963637,"unusualValue":0.12044343,"averageValue":0.05734928,"progressive":1.4422141},{"value":0.3090566,"defaultValue":0.29781818,"unusualValue":0.3090566,"averageValue":0.15452428,"progressive":1.9882141},{"value":0.06735849,"defaultValue":0.06490909,"unusualValue":0.06735849,"averageValue":0.033678368,"progressive":2.1072142},{"value":0.2609434,"defaultValue":0.21276924,"unusualValue":0.2609434,"averageValue":0.13046831,"progressive":2.5682142},{"value":0.14660378,"defaultValue":0.119538456,"unusualValue":0.14660378,"averageValue":0.07329998,"progressive":2.8272142},{"value":0.0356978,"defaultValue":0.029076923,"unusualValue":0.03566038,"averageValue":0.017829726,"progressive":2.8902142},{"value":0.15962264,"defaultValue":0.188,"unusualValue":0.15962264,"averageValue":0.07963559,"progressive":3.1722143},{"value":0.027169812,"defaultValue":0.032,"unusualValue":0.027169812,"averageValue":0.013540026,"progressive":3.2202144},{"value":0.20004307,"defaultValue":0.23533332,"unusualValue":0.19981131,"averageValue":0.0995756,"progressive":3.5732143},{"value":0.07209581,"defaultValue":0.085999995,"unusualValue":0.073018864,"averageValue":0.03638882,"progressive":3.7022142},{"value":0.016981132,"defaultValue":0.02,"unusualValue":0.016981132,"averageValue":0.008462516,"progressive":3.7322142},{"value":0.06905661,"defaultValue":0.08133334,"unusualValue":0.06905661,"averageValue":0.03441423,"progressive":3.8542142},{"value":0.03283019,"defaultValue":0.038666666,"unusualValue":0.03283019,"averageValue":0.016360864,"progressive":3.9122143},{"value":0.23046982,"defaultValue":0.26933336,"unusualValue":0.22867925,"averageValue":0.11396188,"progressive":4.316214},{"value":0.068490565,"defaultValue":0.08066667,"unusualValue":0.068490565,"averageValue":0.03416988,"progressive":4.437214},{"value":0.28740928,"defaultValue":0.33800003,"unusualValue":0.28698114,"averageValue":0.14301652,"progressive":4.944214},{"value":0.032236435,"defaultValue":0.02676923,"unusualValue":0.031926606,"averageValue":0.015931344,"progressive":5.002214},{"value":0.024770644,"defaultValue":0.020769231,"unusualValue":0.024770644,"averageValue":0.012367469,"progressive":5.047214},{"value":0.059999995,"defaultValue":0.05030769,"unusualValue":0.059999995,"averageValue":0.029939938,"progressive":5.156214},{"value":0.052844036,"defaultValue":0.044307694,"unusualValue":0.052844036,"averageValue":0.02636912,"progressive":5.2522144},{"value":0.01531915,"defaultValue":0.012923078,"unusualValue":0.015412845,"averageValue":0.007690994,"progressive":5.2802143},{"value":0.030275228,"defaultValue":0.025384614,"unusualValue":0.030275228,"averageValue":0.0151073085,"progressive":5.335214},{"value":0.0679797,"defaultValue":0.05723077,"unusualValue":0.068256885,"averageValue":0.034060117,"progressive":5.459214},{"value":0.005492958,"defaultValue":0.0046153846,"unusualValue":0.005504587,"averageValue":0.0027467834,"progressive":5.4692144},{"value":0.045137618,"defaultValue":0.037846155,"unusualValue":0.045137618,"averageValue":0.045072556,"progressive":5.551214},{"value":0.066836044,"defaultValue":0.056307696,"unusualValue":0.067155965,"averageValue":0.06702152,"progressive":5.6732144},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.009339064,"progressive":5.6902146},{"value":0.29669726,"defaultValue":0.24876921,"unusualValue":0.29669726,"averageValue":0.29610327,"progressive":6.2292147},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.009339064,"progressive":6.246215},{"value":0.18,"defaultValue":0.15092307,"unusualValue":0.18,"averageValue":0.17963965,"progressive":6.573215},{"value":0.0814679,"defaultValue":0.06830769,"unusualValue":0.0814679,"averageValue":0.081304796,"progressive":6.7212152},{"value":0.006055046,"defaultValue":0.005076923,"unusualValue":0.006055046,"averageValue":0.006042924,"progressive":6.7322154},{"value":0.080235526,"defaultValue":0.067384616,"unusualValue":0.08036697,"averageValue":0.080206074,"progressive":6.8782153},{"value":0.058348626,"defaultValue":0.048923075,"unusualValue":0.058348626,"averageValue":0.058231812,"progressive":6.9842153},{"value":0.20311926,"defaultValue":0.17030768,"unusualValue":0.20311926,"averageValue":0.20271263,"progressive":7.353215},{"value":0.0066055045,"defaultValue":0.0055384617,"unusualValue":0.0066055045,"averageValue":0.00659228,"progressive":7.3652153},{"value":0.04293578,"defaultValue":0.036000002,"unusualValue":0.04293578,"averageValue":0.042873893,"progressive":7.4432154},{"value":0.041553956,"defaultValue":0.035076924,"unusualValue":0.04183486,"averageValue":0.04175111,"progressive":7.5192156},{"value":0.3253211,"defaultValue":0.27276924,"unusualValue":0.3253211,"avera...</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:40:18.535Z</t>
+  </si>
+  <si>
+    <t>Success: Added 17 rows to KPI_list table</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:56:46.333Z</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:56:46.840Z</t>
+  </si>
+  <si>
+    <t>[{"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","timeStamp":"2025-04-07T14:47:00Z","results":[{"value":0.702574,"defaultValue":0.67702585,"unusualValue":0.702574,"averageValue":0.351287,"progressive":1.2412142},{"value":0.11940594,"defaultValue":0.10963637,"unusualValue":0.113773584,"averageValue":0.056886792,"progressive":1.4422141},{"value":0.3090566,"defaultValue":0.29781818,"unusualValue":0.3090566,"averageValue":0.1545283,"progressive":1.9882141},{"value":0.06735849,"defaultValue":0.06490909,"unusualValue":0.06735849,"averageValue":0.033679243,"progressive":2.1072142},{"value":0.2609434,"defaultValue":0.21276924,"unusualValue":0.2609434,"averageValue":0.1304717,"progressive":2.5682142},{"value":0.14660378,"defaultValue":0.119538456,"unusualValue":0.14660378,"averageValue":0.07330189,"progressive":2.8272142},{"value":0.03568966,"defaultValue":0.029076923,"unusualValue":0.03566038,"averageValue":0.01783019,"progressive":2.8902142},{"value":0.15962264,"defaultValue":0.188,"unusualValue":0.15962264,"averageValue":0.07981132,"progressive":3.1722143},{"value":0.027169812,"defaultValue":0.032,"unusualValue":0.027169812,"averageValue":0.013584906,"progressive":3.2202144},{"value":0.19998284,"defaultValue":0.23533332,"unusualValue":0.19981131,"averageValue":0.099905655,"progressive":3.5732143},{"value":0.073018864,"defaultValue":0.085999995,"unusualValue":0.073018864,"averageValue":0.036509432,"progressive":3.7022142},{"value":0.016981132,"defaultValue":0.02,"unusualValue":0.016981132,"averageValue":0.008490566,"progressive":3.7322142},{"value":0.06905661,"defaultValue":0.08133334,"unusualValue":0.06905661,"averageValue":0.034528304,"progressive":3.8542142},{"value":0.03283019,"defaultValue":0.038666666,"unusualValue":0.03283019,"averageValue":0.016415095,"progressive":3.9122143},{"value":0.23004995,"defaultValue":0.26933336,"unusualValue":0.22867925,"averageValue":0.11433963,"progressive":4.316214},{"value":0.0686322,"defaultValue":0.08066667,"unusualValue":0.068490565,"averageValue":0.034245282,"progressive":4.437214},{"value":0.28698114,"defaultValue":0.33800003,"unusualValue":0.28698114,"averageValue":0.14349057,"progressive":4.944214},{"value":0.031926606,"defaultValue":0.02676923,"unusualValue":0.031926606,"averageValue":0.015891396,"progressive":5.002214},{"value":0.024770644,"defaultValue":0.020769231,"unusualValue":0.024770644,"averageValue":0.01234193,"progressive":5.047214},{"value":0.059999995,"defaultValue":0.05030769,"unusualValue":0.059999995,"averageValue":0.029894892,"progressive":5.156214},{"value":0.052844036,"defaultValue":0.044307694,"unusualValue":0.052844036,"averageValue":0.026329448,"progressive":5.2522144},{"value":0.015412845,"defaultValue":0.012923078,"unusualValue":0.015412845,"averageValue":0.007679423,"progressive":5.2802143},{"value":0.030275228,"defaultValue":0.025384614,"unusualValue":0.030275228,"averageValue":0.01508458,"progressive":5.335214},{"value":0.068103425,"defaultValue":0.05723077,"unusualValue":0.068256885,"averageValue":0.03400887,"progressive":5.459214},{"value":0.005504587,"defaultValue":0.0046153846,"unusualValue":0.005504587,"averageValue":0.002742651,"progressive":5.4692144},{"value":0.045137618,"defaultValue":0.037846155,"unusualValue":0.045137618,"averageValue":0.044979475,"progressive":5.551214},{"value":0.067155965,"defaultValue":0.056307696,"unusualValue":0.067155965,"averageValue":0.06692068,"progressive":5.6732144},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.0093250135,"progressive":5.6902146},{"value":0.29669726,"defaultValue":0.24876921,"unusualValue":0.29669726,"averageValue":0.29565778,"progressive":6.2292147},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.0093250135,"progressive":6.246215},{"value":0.17806011,"defaultValue":0.15092307,"unusualValue":0.18,"averageValue":0.17936938,"progressive":6.573215},{"value":0.0814679,"defaultValue":0.06830769,"unusualValue":0.0814679,"averageValue":0.08118247,"progressive":6.7212152},{"value":0.006055046,"defaultValue":0.005076923,"unusualValue":0.006055046,"averageValue":0.0060338317,"progressive":6.7322154},{"value":0.08036697,"defaultValue":0.067384616,"unusualValue":0.08036697,"averageValue":0.080085404,"progressive":6.8782153},{"value":0.058348626,"defaultValue":0.048923075,"unusualValue":0.058348626,"averageValue":0.0581442,"progressive":6.9842153},{"value":0.20311926,"defaultValue":0.17030768,"unusualValue":0.20311926,"averageValue":0.20240763,"progressive":7.353215},{"value":0.0066055045,"defaultValue":0.0055384617,"unusualValue":0.0066055045,"averageValue":0.006582362,"progressive":7.3652153},{"value":0.04293578,"defaultValue":0.036000002,"unusualValue":0.04293578,"averageValue":0.042785354,"progressive":7.4432154},{"value":0.041517448,"defaultValue":0.035076924,"unusualValue":0.04183486,"averageValue":0.041688293,"progressive":7.5192156},{"value":0.3253211,"defaultValue":0.27276924,"unusualValue":0.3253211,"...</t>
+  </si>
+  <si>
+    <t>2025-04-07T14:56:48.968Z</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">IN </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>orange</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : cells THAT CAN BE EDITED BY THE USER</t>
+    </r>
+  </si>
+  <si>
+    <t>apiKey</t>
+  </si>
+  <si>
+    <t>fromTime (ISO 8601 format) UTC</t>
+  </si>
+  <si>
+    <t>toTime (ISO 8601 format) UTC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,6 +401,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -394,21 +447,31 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -501,6 +564,26 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -530,86 +613,161 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <font>
         <sz val="11"/>
@@ -642,6 +800,32 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -893,7 +1077,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-US"/>
-            <a:t>Get overall Kpi</a:t>
+            <a:t>Get HDA overall Kpi</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" baseline="0"/>
@@ -1069,15 +1253,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>171450</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>409575</xdr:rowOff>
+      <xdr:rowOff>400050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1047751</xdr:colOff>
+      <xdr:colOff>1095376</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1095,7 +1279,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4838700" y="2609850"/>
+          <a:off x="4886325" y="2600325"/>
           <a:ext cx="2638426" cy="390525"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -1212,9 +1396,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>171450</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>90488</xdr:rowOff>
+      <xdr:rowOff>80963</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1233,7 +1417,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4445000" y="1889125"/>
-          <a:ext cx="393700" cy="915988"/>
+          <a:ext cx="441325" cy="906463"/>
         </a:xfrm>
         <a:prstGeom prst="curvedConnector3">
           <a:avLst>
@@ -1439,9 +1623,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>847725</xdr:colOff>
+      <xdr:colOff>876300</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
+      <xdr:rowOff>171449</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1457,7 +1641,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="847725" y="1343024"/>
+          <a:off x="876300" y="1704974"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -1776,10 +1960,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>123824</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2400300</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47624</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="361950" cy="332003"/>
     <xdr:sp macro="" textlink="">
@@ -1795,7 +1979,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2505075" y="1276349"/>
+          <a:off x="2400300" y="1771649"/>
           <a:ext cx="361950" cy="332003"/>
         </a:xfrm>
         <a:custGeom>
@@ -2760,16 +2944,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>771524</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>485774</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>171449</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1866900</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2787,8 +2971,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9715499" y="1724025"/>
-          <a:ext cx="1628775" cy="666750"/>
+          <a:off x="8505824" y="1685925"/>
+          <a:ext cx="2305051" cy="666750"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2841,32 +3025,34 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Luca PAONE (PTV Group)" id="{FE2F6ED8-9348-4908-88B0-71F732C27369}" userId="S::luca.paone@ptvgroup.com::33599286-32ca-48eb-a86d-fc71f4f812d2" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F21" insertRow="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F22" insertRow="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="18" totalsRowDxfId="19">
   <autoFilter ref="A20:F21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID"/>
-    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name"/>
-    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name"/>
-    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID"/>
-    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Length (km)"/>
-    <tableColumn id="6" xr3:uid="{A51E7A9B-B66E-4276-B542-A89F10024F5B}" name="KPI url" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="16" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="15" totalsRowDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="14" totalsRowDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="13" totalsRowDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="12" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{CEC8F276-428E-4168-BCEA-8D77F1D4A8F0}" name="RequestLog" displayName="RequestLog" ref="A1:D2" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:D2" xr:uid="{CEC8F276-428E-4168-BCEA-8D77F1D4A8F0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}" name="RequestLog" displayName="RequestLog" ref="A1:D12" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:D12" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{F7903956-1621-4950-8968-28984C0E493E}" name="Datetime" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{7A66C07F-4972-440B-9EE8-5889126D5746}" name="Request URL" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{BE6CC200-999E-4F58-B832-0DC74CBFC9DB}" name="Status" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{DA42A551-1F18-43DE-8E76-DFA72E495F64}" name="Body (answer)" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{94788DBD-DB73-4499-9554-13FD83D56E99}" name="Datetime" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{1B49E132-7BC4-47FA-B194-A8662469036D}" name="Request URL" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{EFFC061F-6CE6-47DD-B6F4-8B601FE36300}" name="Status" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{8A164B4F-6F22-4123-A5F9-CE61462B18B6}" name="Body (answer)" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3133,6 +3319,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B5" dT="2025-04-07T15:11:20.63" personId="{FE2F6ED8-9348-4908-88B0-71F732C27369}" id="{248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}">
+    <text>Attention, Time and Date in UTC</text>
+  </threadedComment>
+  <threadedComment ref="C5" dT="2025-04-07T15:11:28.96" personId="{FE2F6ED8-9348-4908-88B0-71F732C27369}" id="{B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}">
+    <text>Attention, Time and Date in UTC</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="4">
@@ -3150,407 +3347,1248 @@
   <we:properties/>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
 </we:webextension>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G172"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K296"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
     <col min="4" max="4" width="23.85546875" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
     <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="20" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="30" t="str">
+        <f>TEXT(B4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B5, "HH:MM:SS") &amp; "Z"</f>
+        <v>2025-03-01T00:00:00Z</v>
+      </c>
+      <c r="C3" s="31" t="str">
+        <f>TEXT(C4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C5, "HH:MM:SS") &amp; "Z"</f>
+        <v>2025-03-01T23:59:00Z</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="17">
+        <v>45717</v>
+      </c>
+      <c r="C4" s="17">
+        <v>45717</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="19">
+        <v>0</v>
+      </c>
+      <c r="C5" s="19">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E9" s="4"/>
-    </row>
-    <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E11" s="2"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E17" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="16"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="23"/>
+      <c r="G17" s="24"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E18" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20" t="s">
-        <v>3</v>
-      </c>
-      <c r="C20" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" t="s">
-        <v>5</v>
-      </c>
-      <c r="E20" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20" t="s">
-        <v>52</v>
-      </c>
+      <c r="A20" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="11"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F21" s="13"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="28"/>
+      <c r="G21" s="29"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F22" s="13"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="11"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F23" s="13"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F24" s="13"/>
+      <c r="A24" s="27"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="11"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F25" s="13"/>
+      <c r="A25" s="27"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="11"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F26" s="13"/>
+      <c r="A26" s="27"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="11"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F27" s="13"/>
+      <c r="A27" s="27"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="11"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F28" s="13"/>
+      <c r="A28" s="27"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="11"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="F29" s="13"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="11"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="F30" s="13"/>
+      <c r="A30" s="27"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="11"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="F31" s="13"/>
+      <c r="A31" s="27"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="11"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="F32" s="13"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-      <c r="F33" s="13"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="F34" s="13"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
-      <c r="F35" s="13"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
-      <c r="F36" s="13"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="F37" s="13"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
-      <c r="F38" s="13"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-      <c r="F39" s="13"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="1"/>
-      <c r="F40" s="13"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-      <c r="F41" s="13"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-      <c r="F42" s="13"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="1"/>
-      <c r="F43" s="13"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1"/>
-      <c r="F44" s="13"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
-      <c r="F45" s="13"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="1"/>
-      <c r="F46" s="13"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1"/>
-      <c r="F47" s="13"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="1"/>
-      <c r="F48" s="13"/>
+      <c r="A32" s="27"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="11"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="27"/>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="11"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="27"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="11"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="27"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="11"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="27"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="28"/>
+      <c r="G36" s="11"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="27"/>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="27"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="11"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="27"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="11"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="27"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="27"/>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="28"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="27"/>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="28"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="27"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
+      <c r="F43" s="28"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="27"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="28"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="27"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="28"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="27"/>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="28"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="27"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="28"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="27"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="28"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
-      <c r="F49" s="13"/>
+      <c r="A49" s="27"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="28"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="1"/>
-      <c r="F50" s="13"/>
+      <c r="A50" s="27"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="28"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
-      <c r="F51" s="13"/>
+      <c r="A51" s="27"/>
+      <c r="B51" s="11"/>
+      <c r="C51" s="11"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="28"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="1"/>
-      <c r="F52" s="13"/>
+      <c r="A52" s="27"/>
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="28"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="1"/>
-      <c r="F53" s="13"/>
+      <c r="A53" s="27"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="28"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="1"/>
-      <c r="F54" s="13"/>
+      <c r="A54" s="27"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="28"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="1"/>
+      <c r="A55" s="27"/>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="28"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
+      <c r="A56" s="11"/>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="28"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="1"/>
+      <c r="A57" s="27"/>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="28"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
+      <c r="F58" s="6"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
+      <c r="F59" s="6"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
+      <c r="F60" s="6"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
+      <c r="F61" s="6"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
+      <c r="F62" s="6"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
+      <c r="F63" s="6"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F64" s="6"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F65" s="6"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F66" s="6"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F67" s="6"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F68" s="6"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F69" s="6"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F70" s="6"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F71" s="6"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="1"/>
+      <c r="F72" s="6"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="1"/>
+      <c r="F73" s="6"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="1"/>
+      <c r="F74" s="6"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="1"/>
+      <c r="F75" s="6"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="1"/>
+      <c r="F76" s="6"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="1"/>
+      <c r="F77" s="6"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="1"/>
+      <c r="F78" s="6"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F79" s="6"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F80" s="6"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F81" s="6"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F82" s="6"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F83" s="6"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F84" s="6"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F85" s="6"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F86" s="6"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F87" s="6"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="1"/>
+      <c r="F88" s="6"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="1"/>
+      <c r="F89" s="6"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="1"/>
+      <c r="F90" s="6"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="1"/>
+      <c r="F91" s="6"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="1"/>
+      <c r="F92" s="6"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="1"/>
+      <c r="F93" s="6"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="1"/>
+      <c r="F94" s="6"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F95" s="6"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F96" s="6"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F97" s="6"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F98" s="6"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F99" s="6"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F100" s="6"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F101" s="6"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F102" s="6"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F103" s="6"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="1"/>
+      <c r="F104" s="6"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="1"/>
+      <c r="F105" s="6"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="1"/>
+      <c r="F106" s="6"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="1"/>
+      <c r="F107" s="6"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="1"/>
+      <c r="F108" s="6"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="1"/>
+      <c r="F109" s="6"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="1"/>
+      <c r="F110" s="6"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="1"/>
+      <c r="F111" s="6"/>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F112" s="6"/>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="1"/>
+      <c r="F113" s="6"/>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" s="1"/>
+      <c r="F114" s="6"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" s="1"/>
+      <c r="F115" s="6"/>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" s="1"/>
+      <c r="F116" s="6"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" s="1"/>
+      <c r="F117" s="6"/>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" s="1"/>
+      <c r="F118" s="6"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" s="1"/>
+      <c r="F119" s="6"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" s="1"/>
+      <c r="F120" s="6"/>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" s="1"/>
+      <c r="F121" s="6"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" s="1"/>
+      <c r="F122" s="6"/>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" s="1"/>
+      <c r="F123" s="6"/>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="1"/>
+      <c r="F124" s="6"/>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" s="1"/>
+      <c r="F125" s="6"/>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A126" s="1"/>
+      <c r="F126" s="6"/>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" s="1"/>
+      <c r="F127" s="6"/>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F128" s="6"/>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F129" s="6"/>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F130" s="6"/>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F131" s="6"/>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F132" s="6"/>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F133" s="6"/>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F134" s="6"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F135" s="6"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="1"/>
+      <c r="F136" s="6"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" s="1"/>
+      <c r="F137" s="6"/>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" s="1"/>
+      <c r="F138" s="6"/>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" s="1"/>
+      <c r="F139" s="6"/>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" s="1"/>
+      <c r="F140" s="6"/>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" s="1"/>
+      <c r="F141" s="6"/>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" s="1"/>
+      <c r="F142" s="6"/>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" s="1"/>
+      <c r="F143" s="6"/>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F144" s="6"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" s="1"/>
+      <c r="F145" s="6"/>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" s="1"/>
+      <c r="F146" s="6"/>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A147" s="1"/>
+      <c r="F147" s="6"/>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A148" s="1"/>
+      <c r="F148" s="6"/>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A149" s="1"/>
+      <c r="F149" s="6"/>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A150" s="1"/>
+      <c r="F150" s="6"/>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A151" s="1"/>
+      <c r="F151" s="6"/>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A152" s="1"/>
+      <c r="F152" s="6"/>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A153" s="1"/>
+      <c r="F153" s="6"/>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A154" s="1"/>
+      <c r="F154" s="6"/>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A155" s="1"/>
+      <c r="F155" s="6"/>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A156" s="1"/>
+      <c r="F156" s="6"/>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A157" s="1"/>
+      <c r="F157" s="6"/>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A158" s="1"/>
+      <c r="F158" s="6"/>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A159" s="1"/>
+      <c r="F159" s="6"/>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A160" s="1"/>
+      <c r="F160" s="6"/>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A161" s="1"/>
+      <c r="F161" s="6"/>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A162" s="1"/>
+      <c r="F162" s="6"/>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A163" s="1"/>
+      <c r="F163" s="6"/>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A164" s="1"/>
+      <c r="F164" s="6"/>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A165" s="1"/>
+      <c r="F165" s="6"/>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A166" s="1"/>
+      <c r="F166" s="6"/>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A167" s="1"/>
+      <c r="F167" s="6"/>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" s="1"/>
+      <c r="F168" s="6"/>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" s="1"/>
+      <c r="F169" s="6"/>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" s="1"/>
+      <c r="F170" s="6"/>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="1"/>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F171" s="6"/>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
     </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" s="1"/>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" s="1"/>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" s="1"/>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" s="1"/>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A177" s="1"/>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A178" s="1"/>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A179" s="1"/>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A180" s="1"/>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A181" s="1"/>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A182" s="1"/>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A183" s="1"/>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A184" s="1"/>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A185" s="1"/>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A186" s="1"/>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A187" s="1"/>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A188" s="1"/>
+      <c r="F188" s="6"/>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A189" s="1"/>
+      <c r="F189" s="6"/>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A190" s="1"/>
+      <c r="F190" s="6"/>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A191" s="1"/>
+      <c r="F191" s="6"/>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A192" s="1"/>
+      <c r="F192" s="6"/>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A193" s="1"/>
+      <c r="F193" s="6"/>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A194" s="1"/>
+      <c r="F194" s="6"/>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A195" s="1"/>
+      <c r="F195" s="6"/>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F196" s="6"/>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F197" s="6"/>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F198" s="6"/>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F199" s="6"/>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F200" s="6"/>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F201" s="6"/>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F202" s="6"/>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A203" s="1"/>
+      <c r="F203" s="6"/>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A204" s="1"/>
+      <c r="F204" s="6"/>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A205" s="1"/>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A206" s="1"/>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A207" s="1"/>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A208" s="1"/>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209" s="1"/>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210" s="1"/>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211" s="1"/>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219" s="1"/>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220" s="1"/>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221" s="1"/>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222" s="1"/>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223" s="1"/>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224" s="1"/>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" s="1"/>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226" s="1"/>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227" s="1"/>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236" s="1"/>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" s="1"/>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" s="1"/>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295" s="1"/>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296" s="1"/>
+    </row>
   </sheetData>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="2">
+    <mergeCell ref="E18:G18"/>
     <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E18:G18"/>
   </mergeCells>
+  <phoneticPr fontId="10" type="noConversion"/>
+  <dataValidations count="4">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a correct date" error="please input a correct date_x000a_" sqref="B4:C4" xr:uid="{F83F3375-2F4B-4A5A-9230-C8D6497346A1}">
+      <formula1>45658</formula1>
+      <formula2>47484</formula2>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5:C5" xr:uid="{B6FD0E10-0D6F-44F3-B446-DA33EADAEAEB}">
+      <formula1>0</formula1>
+      <formula2>0.999305555555556</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3" xr:uid="{9367E08E-DE83-4A16-AE23-738728604C7E}">
+      <formula1>$D$4:$D$8</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:C3" xr:uid="{5AD50032-6A28-44BB-BCD8-0C40654E1CEC}">
+      <formula1>AND(ISNUMBER(FIND("T", A1)), ISNUMBER(FIND("Z", A1)), LEN(A1)=20, ISNUMBER(DATEVALUE(LEFT(A1, 10))), ISNUMBER(TIMEVALUE(MID(A1, 12, 8))))</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -3560,24 +4598,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="19" t="s">
-        <v>37</v>
+      <c r="A1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3590,150 +4760,130 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A57C2C16-3654-4C73-B5DD-4EE8172FF9A3}">
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>39</v>
+      <c r="A1" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>40</v>
+      <c r="A2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>44</v>
+      <c r="A7" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>19</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>21</v>
+      <c r="A15" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>46</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>48</v>
-      </c>
+      <c r="A26" s="2"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>49</v>
+      <c r="A27" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>26</v>
+      <c r="A31" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3742,26 +4892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -3990,7 +5120,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
@@ -4003,32 +5133,27 @@
 </scriptIds>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="43744f66-d8c7-4420-ad58-b4d72814d14f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4047,11 +5172,30 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
     <ds:schemaRef ds:uri=""/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
+    <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
corrected header of km length for GetLocation script
corrected header of km length for GetLocation script
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95DDA57B-3676-45BB-A66F-CCDE6B669731}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{919CF4C8-5B92-4BCF-9328-32B3F3178D96}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -374,10 +374,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -466,12 +466,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -619,19 +613,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
@@ -665,14 +652,14 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -681,6 +668,32 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -695,36 +708,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -732,42 +715,6 @@
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="21">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="15" formatCode="0.00E+00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
     <dxf>
       <font>
         <sz val="11"/>
@@ -799,6 +746,26 @@
       </font>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -812,6 +779,22 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -3031,28 +3014,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F22" insertRow="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="18" totalsRowDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F22" insertRow="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="18">
   <autoFilter ref="A20:F21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="16" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="15" totalsRowDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="14" totalsRowDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="13" totalsRowDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="12" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}" name="RequestLog" displayName="RequestLog" ref="A1:D12" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}" name="RequestLog" displayName="RequestLog" ref="A1:D12" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A1:D12" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{94788DBD-DB73-4499-9554-13FD83D56E99}" name="Datetime" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{1B49E132-7BC4-47FA-B194-A8662469036D}" name="Request URL" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{EFFC061F-6CE6-47DD-B6F4-8B601FE36300}" name="Status" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{8A164B4F-6F22-4123-A5F9-CE61462B18B6}" name="Body (answer)" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{94788DBD-DB73-4499-9554-13FD83D56E99}" name="Datetime" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{1B49E132-7BC4-47FA-B194-A8662469036D}" name="Request URL" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{EFFC061F-6CE6-47DD-B6F4-8B601FE36300}" name="Status" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{8A164B4F-6F22-4123-A5F9-CE61462B18B6}" name="Body (answer)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3357,7 +3340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K296"/>
+  <dimension ref="A1:G296"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -3372,1014 +3355,1012 @@
     <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="K1" s="5"/>
-    </row>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+    </row>
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="30" t="str">
+      <c r="B3" s="22" t="str">
         <f>TEXT(B4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B5, "HH:MM:SS") &amp; "Z"</f>
         <v>2025-03-01T00:00:00Z</v>
       </c>
-      <c r="C3" s="31" t="str">
+      <c r="C3" s="23" t="str">
         <f>TEXT(C4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C5, "HH:MM:SS") &amp; "Z"</f>
         <v>2025-03-01T23:59:00Z</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+    </row>
+    <row r="4" spans="1:7" ht="30.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="14">
         <v>45717</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="14">
         <v>45717</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-    </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+    </row>
+    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="16">
         <v>0</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="16">
         <v>0.99930555555555556</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11" t="s">
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11" t="s">
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11" t="s">
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-    </row>
-    <row r="10" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-    </row>
-    <row r="11" spans="1:11" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+    </row>
+    <row r="10" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="22" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="24"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="29"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
       <c r="E18" s="25"/>
       <c r="F18" s="26"/>
       <c r="G18" s="26"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G20" s="11"/>
+      <c r="G20" s="8"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="27"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="29"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="21"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="27"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="11"/>
+      <c r="A22" s="19"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="27"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="11"/>
+      <c r="A23" s="19"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="8"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="27"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="11"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="27"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="11"/>
+      <c r="A25" s="19"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="8"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="27"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="11"/>
+      <c r="A26" s="19"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="27"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="11"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="8"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="27"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="11"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="8"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="27"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="11"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="8"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="27"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="11"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="27"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="11"/>
+      <c r="A31" s="19"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="8"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="27"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="11"/>
+      <c r="A32" s="19"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="27"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="11"/>
+      <c r="A33" s="19"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="8"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="27"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="28"/>
-      <c r="G34" s="11"/>
+      <c r="A34" s="19"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="8"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="27"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="11"/>
+      <c r="A35" s="19"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="8"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="27"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="28"/>
-      <c r="G36" s="11"/>
+      <c r="A36" s="19"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="27"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="11"/>
+      <c r="A37" s="19"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="8"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="27"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="11"/>
+      <c r="A38" s="19"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="27"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="11"/>
+      <c r="A39" s="19"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="8"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="27"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="11"/>
+      <c r="A40" s="19"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="8"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="27"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="28"/>
+      <c r="A41" s="19"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="20"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="27"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="28"/>
+      <c r="A42" s="19"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="20"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="27"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="28"/>
+      <c r="A43" s="19"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="20"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="27"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="28"/>
+      <c r="A44" s="19"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="20"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="27"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="28"/>
+      <c r="A45" s="19"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="20"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="27"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="28"/>
+      <c r="A46" s="19"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="20"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="27"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="28"/>
+      <c r="A47" s="19"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="20"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="27"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="28"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="20"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="27"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="28"/>
+      <c r="A49" s="19"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="20"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="27"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="28"/>
+      <c r="A50" s="19"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="20"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="27"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="28"/>
+      <c r="A51" s="19"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="20"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="27"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="28"/>
+      <c r="A52" s="19"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="20"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="27"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="28"/>
+      <c r="A53" s="19"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="20"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="27"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="28"/>
+      <c r="A54" s="19"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="20"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="27"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="28"/>
+      <c r="A55" s="19"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="20"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="28"/>
+      <c r="A56" s="8"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="20"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="27"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="28"/>
+      <c r="A57" s="19"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="20"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
-      <c r="F58" s="6"/>
+      <c r="F58" s="4"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
-      <c r="F59" s="6"/>
+      <c r="F59" s="4"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
-      <c r="F60" s="6"/>
+      <c r="F60" s="4"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
-      <c r="F61" s="6"/>
+      <c r="F61" s="4"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
-      <c r="F62" s="6"/>
+      <c r="F62" s="4"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
-      <c r="F63" s="6"/>
+      <c r="F63" s="4"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
-      <c r="F64" s="6"/>
+      <c r="F64" s="4"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
-      <c r="F65" s="6"/>
+      <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
-      <c r="F66" s="6"/>
+      <c r="F66" s="4"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
-      <c r="F67" s="6"/>
+      <c r="F67" s="4"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
-      <c r="F68" s="6"/>
+      <c r="F68" s="4"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
-      <c r="F69" s="6"/>
+      <c r="F69" s="4"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
-      <c r="F70" s="6"/>
+      <c r="F70" s="4"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
-      <c r="F71" s="6"/>
+      <c r="F71" s="4"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
-      <c r="F72" s="6"/>
+      <c r="F72" s="4"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
-      <c r="F73" s="6"/>
+      <c r="F73" s="4"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
-      <c r="F74" s="6"/>
+      <c r="F74" s="4"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
-      <c r="F75" s="6"/>
+      <c r="F75" s="4"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
-      <c r="F76" s="6"/>
+      <c r="F76" s="4"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
-      <c r="F77" s="6"/>
+      <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
-      <c r="F78" s="6"/>
+      <c r="F78" s="4"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
-      <c r="F79" s="6"/>
+      <c r="F79" s="4"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
-      <c r="F80" s="6"/>
+      <c r="F80" s="4"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
-      <c r="F81" s="6"/>
+      <c r="F81" s="4"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
-      <c r="F82" s="6"/>
+      <c r="F82" s="4"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
-      <c r="F83" s="6"/>
+      <c r="F83" s="4"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
-      <c r="F84" s="6"/>
+      <c r="F84" s="4"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
-      <c r="F85" s="6"/>
+      <c r="F85" s="4"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
-      <c r="F86" s="6"/>
+      <c r="F86" s="4"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
-      <c r="F87" s="6"/>
+      <c r="F87" s="4"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
-      <c r="F88" s="6"/>
+      <c r="F88" s="4"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
-      <c r="F89" s="6"/>
+      <c r="F89" s="4"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
-      <c r="F90" s="6"/>
+      <c r="F90" s="4"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
-      <c r="F91" s="6"/>
+      <c r="F91" s="4"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
-      <c r="F92" s="6"/>
+      <c r="F92" s="4"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
-      <c r="F93" s="6"/>
+      <c r="F93" s="4"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
-      <c r="F94" s="6"/>
+      <c r="F94" s="4"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
-      <c r="F95" s="6"/>
+      <c r="F95" s="4"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
-      <c r="F96" s="6"/>
+      <c r="F96" s="4"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
-      <c r="F97" s="6"/>
+      <c r="F97" s="4"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
-      <c r="F98" s="6"/>
+      <c r="F98" s="4"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
-      <c r="F99" s="6"/>
+      <c r="F99" s="4"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
-      <c r="F100" s="6"/>
+      <c r="F100" s="4"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
-      <c r="F101" s="6"/>
+      <c r="F101" s="4"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
-      <c r="F102" s="6"/>
+      <c r="F102" s="4"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
-      <c r="F103" s="6"/>
+      <c r="F103" s="4"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
-      <c r="F104" s="6"/>
+      <c r="F104" s="4"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
-      <c r="F105" s="6"/>
+      <c r="F105" s="4"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
-      <c r="F106" s="6"/>
+      <c r="F106" s="4"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
-      <c r="F107" s="6"/>
+      <c r="F107" s="4"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
-      <c r="F108" s="6"/>
+      <c r="F108" s="4"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
-      <c r="F109" s="6"/>
+      <c r="F109" s="4"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
-      <c r="F110" s="6"/>
+      <c r="F110" s="4"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
-      <c r="F111" s="6"/>
+      <c r="F111" s="4"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
-      <c r="F112" s="6"/>
+      <c r="F112" s="4"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
-      <c r="F113" s="6"/>
+      <c r="F113" s="4"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
-      <c r="F114" s="6"/>
+      <c r="F114" s="4"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
-      <c r="F115" s="6"/>
+      <c r="F115" s="4"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
-      <c r="F116" s="6"/>
+      <c r="F116" s="4"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
-      <c r="F117" s="6"/>
+      <c r="F117" s="4"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
-      <c r="F118" s="6"/>
+      <c r="F118" s="4"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
-      <c r="F119" s="6"/>
+      <c r="F119" s="4"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
-      <c r="F120" s="6"/>
+      <c r="F120" s="4"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
-      <c r="F121" s="6"/>
+      <c r="F121" s="4"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
-      <c r="F122" s="6"/>
+      <c r="F122" s="4"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
-      <c r="F123" s="6"/>
+      <c r="F123" s="4"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
-      <c r="F124" s="6"/>
+      <c r="F124" s="4"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
-      <c r="F125" s="6"/>
+      <c r="F125" s="4"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
-      <c r="F126" s="6"/>
+      <c r="F126" s="4"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
-      <c r="F127" s="6"/>
+      <c r="F127" s="4"/>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
-      <c r="F128" s="6"/>
+      <c r="F128" s="4"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F129" s="6"/>
+      <c r="F129" s="4"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F130" s="6"/>
+      <c r="F130" s="4"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F131" s="6"/>
+      <c r="F131" s="4"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F132" s="6"/>
+      <c r="F132" s="4"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F133" s="6"/>
+      <c r="F133" s="4"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F134" s="6"/>
+      <c r="F134" s="4"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F135" s="6"/>
+      <c r="F135" s="4"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
-      <c r="F136" s="6"/>
+      <c r="F136" s="4"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="1"/>
-      <c r="F137" s="6"/>
+      <c r="F137" s="4"/>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="1"/>
-      <c r="F138" s="6"/>
+      <c r="F138" s="4"/>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="1"/>
-      <c r="F139" s="6"/>
+      <c r="F139" s="4"/>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="1"/>
-      <c r="F140" s="6"/>
+      <c r="F140" s="4"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="1"/>
-      <c r="F141" s="6"/>
+      <c r="F141" s="4"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
-      <c r="F142" s="6"/>
+      <c r="F142" s="4"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="1"/>
-      <c r="F143" s="6"/>
+      <c r="F143" s="4"/>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
-      <c r="F144" s="6"/>
+      <c r="F144" s="4"/>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="1"/>
-      <c r="F145" s="6"/>
+      <c r="F145" s="4"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="1"/>
-      <c r="F146" s="6"/>
+      <c r="F146" s="4"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="1"/>
-      <c r="F147" s="6"/>
+      <c r="F147" s="4"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
-      <c r="F148" s="6"/>
+      <c r="F148" s="4"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="1"/>
-      <c r="F149" s="6"/>
+      <c r="F149" s="4"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="1"/>
-      <c r="F150" s="6"/>
+      <c r="F150" s="4"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="1"/>
-      <c r="F151" s="6"/>
+      <c r="F151" s="4"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="1"/>
-      <c r="F152" s="6"/>
+      <c r="F152" s="4"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="1"/>
-      <c r="F153" s="6"/>
+      <c r="F153" s="4"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
-      <c r="F154" s="6"/>
+      <c r="F154" s="4"/>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="1"/>
-      <c r="F155" s="6"/>
+      <c r="F155" s="4"/>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" s="1"/>
-      <c r="F156" s="6"/>
+      <c r="F156" s="4"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" s="1"/>
-      <c r="F157" s="6"/>
+      <c r="F157" s="4"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" s="1"/>
-      <c r="F158" s="6"/>
+      <c r="F158" s="4"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="1"/>
-      <c r="F159" s="6"/>
+      <c r="F159" s="4"/>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
-      <c r="F160" s="6"/>
+      <c r="F160" s="4"/>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
-      <c r="F161" s="6"/>
+      <c r="F161" s="4"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
-      <c r="F162" s="6"/>
+      <c r="F162" s="4"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
-      <c r="F163" s="6"/>
+      <c r="F163" s="4"/>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
-      <c r="F164" s="6"/>
+      <c r="F164" s="4"/>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
-      <c r="F165" s="6"/>
+      <c r="F165" s="4"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
-      <c r="F166" s="6"/>
+      <c r="F166" s="4"/>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="1"/>
-      <c r="F167" s="6"/>
+      <c r="F167" s="4"/>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="1"/>
-      <c r="F168" s="6"/>
+      <c r="F168" s="4"/>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="1"/>
-      <c r="F169" s="6"/>
+      <c r="F169" s="4"/>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="1"/>
-      <c r="F170" s="6"/>
+      <c r="F170" s="4"/>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="1"/>
-      <c r="F171" s="6"/>
+      <c r="F171" s="4"/>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
@@ -4431,64 +4412,64 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
-      <c r="F188" s="6"/>
+      <c r="F188" s="4"/>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
-      <c r="F189" s="6"/>
+      <c r="F189" s="4"/>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
-      <c r="F190" s="6"/>
+      <c r="F190" s="4"/>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
-      <c r="F191" s="6"/>
+      <c r="F191" s="4"/>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
-      <c r="F192" s="6"/>
+      <c r="F192" s="4"/>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
-      <c r="F193" s="6"/>
+      <c r="F193" s="4"/>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
-      <c r="F194" s="6"/>
+      <c r="F194" s="4"/>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
-      <c r="F195" s="6"/>
+      <c r="F195" s="4"/>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F196" s="6"/>
+      <c r="F196" s="4"/>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F197" s="6"/>
+      <c r="F197" s="4"/>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F198" s="6"/>
+      <c r="F198" s="4"/>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F199" s="6"/>
+      <c r="F199" s="4"/>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F200" s="6"/>
+      <c r="F200" s="4"/>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F201" s="6"/>
+      <c r="F201" s="4"/>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F202" s="6"/>
+      <c r="F202" s="4"/>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
-      <c r="F203" s="6"/>
+      <c r="F203" s="4"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
-      <c r="F204" s="6"/>
+      <c r="F204" s="4"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
@@ -4598,156 +4579,146 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-    </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" t="s">
         <v>47</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="7"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4892,6 +4863,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
+</scriptIds>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -5120,28 +5113,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
-</scriptIds>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5154,6 +5125,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5172,23 +5160,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
input with your timezone is now supported (output is always in UTC)
input with your timezone is now supported (output is always in UTC)
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{919CF4C8-5B92-4BCF-9328-32B3F3178D96}"/>
+  <xr:revisionPtr revIDLastSave="551" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{094FED43-8375-4948-BC31-A585458D2D51}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,22 +42,33 @@
   <authors>
     <author>tc={248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}</author>
     <author>tc={B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}</author>
+    <author>tc={716D20F0-8F3A-44D5-9F55-DB8295C640BA}</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0" xr:uid="{248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}">
       <text>
-        <t>[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Attention, Time and Date in UTC</t>
+    Attention, Time and Date in your timezone including DST for doubts go to Time Difference between UTC, Time Zone and the World </t>
       </text>
     </comment>
     <comment ref="C5" authorId="1" shapeId="0" xr:uid="{B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}">
       <text>
-        <t>[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Attention, Time and Date in UTC</t>
+    Attention, Time and Date in your timezone including DST for doubts go to Time Difference between UTC, Time Zone and the World 
+</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="2" shapeId="0" xr:uid="{716D20F0-8F3A-44D5-9F55-DB8295C640BA}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Delta in hours between your timezone including current DST if active and the UTC time, in case of doubts go to  to Time Difference between UTC, Time Zone and the World 
+</t>
       </text>
     </comment>
   </commentList>
@@ -65,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>your apiKey &gt;</t>
   </si>
@@ -273,64 +284,22 @@
     <t>KPI url</t>
   </si>
   <si>
-    <t>https://api.ptvgroup.tech/kpieng/v1/instance/all</t>
-  </si>
-  <si>
-    <t>Success: Retrieved 17 KPIs</t>
-  </si>
-  <si>
-    <t>[{"name":"ETT_+20_on_FCO-Tuscolana","notes":"","kpiInstanceParameters":{"parameters":{"timetostart":1200}},"location":{"name":"FCO-Tuscolana","shape":"LINESTRING (12.268298 41.787941, 12.27342 41.79023, 12.28064 41.79425, 12.28259 41.79533, 12.28786 41.79827, 12.28902 41.7989, 12.29347 41.8014, 12.29597 41.80279, 12.29658 41.80313, 12.29929 41.80467, 12.29976 41.80493, 12.30317 41.80683, 12.30442 41.80752, 12.30472 41.80768, 12.30593 41.80832, 12.30652 41.80859, 12.31006 41.81001, 12.31084 41.81026, 12.3122 41.81065, 12.31543 41.81139, 12.31812 41.81177, 12.31881 41.81184, 12.31935 41.81189, 12.32066 41.812, 12.3218 41.81212, 12.32213 41.81214, 12.32279 41.81221, 12.32427 41.81233, 12.3244 41.81234, 12.32537 41.81243, 12.32683 41.81256, 12.32704 41.81258, 12.3335 41.81316, 12.3337 41.81317, 12.33761 41.81354, 12.33939 41.8137, 12.33952 41.81371, 12.34127 41.81386, 12.34254 41.81398, 12.34696 41.81437, 12.3471 41.81438, 12.34804 41.81447, 12.34895 41.81454, 12.35603 41.81518, 12.36148 41.81567, 12.36213 41.81572, 12.36498 41.81597, 12.36893 41.81632, 12.36941 41.81636, 12.37122 41.81654, 12.37245 41.81655, 12.37293 41.81658, 12.37544 41.81676, 12.37606 41.81682, 12.37629 41.81683, 12.37643 41.81684, 12.37671 41.81687, 12.37845 41.81703, 12.38538 41.81762, 12.38562 41.81764, 12.38774 41.81767, 12.38837 41.81758, 12.38956 41.81718, 12.39186 41.81608, 12.39233 41.81575, 12.3931 41.81508, 12.39347 41.81473, 12.3942 41.81411, 12.39585 41.81295, 12.39789 41.81182, 12.3983 41.81162, 12.39841 41.81158, 12.39901 41.81134, 12.40003 41.81096, 12.40153 41.81055, 12.40264 41.81034, 12.4052 41.80975, 12.40598 41.80957, 12.41072 41.80871, 12.4122 41.80849, 12.41494 41.80811, 12.41591 41.80798, 12.4176 41.80774, 12.41793 41.80768, 12.41841 41.80761, 12.41858 41.80759, 12.4194 41.80747, 12.4198 41.80742, 12.41999 41.80739, 12.42042 41.80732, 12.42077 41.80727, 12.42127 41.80718, 12.42248 41.80688, 12.42457 41.80624, 12.4326 41.80362, 12.43585 41.80298, 12.43625 41.80292, 12.43657 41.80288, 12.43668 41.80287, 12.4393 41.80257, 12.44016 41.80248, 12.4422 41.80223, 12.44434 41.80197, 12.44444 41.80196, 12.44478 41.80192, 12.44502 41.80189, 12.44572 41.8018, 12.446 41.80177, 12.44767 41.80156, 12.44829 41.80148, 12.44984 41.8013, 12.44993 41.80129, 12.45316 41.80087, 12.45358 41.80082, 12.45374 41.8008, 12.45395 41.80078, 12.45417 41.80075, 12.4566 41.80046, 12.45748 41.80034, 12.45831 41.80024, 12.4593 41.80012, 12.46124 41.79989, 12.46577 41.79934, 12.4714 41.79865, 12.47545 41.79816, 12.47559 41.79814, 12.47575 41.79812, 12.47604 41.7981, 12.47643 41.79805, 12.47708 41.79796, 12.48015 41.79759, 12.48065 41.79753, 12.48079 41.79752, 12.48097 41.79749, 12.48126 41.79746, 12.48422 41.7971, 12.48461 41.79705, 12.48558 41.79693, 12.49026 41.79636, 12.49957 41.79525, 12.50449 41.79465, 12.50705 41.79433, 12.50787 41.79425, 12.50835 41.79421, 12.51102 41.79412, 12.51118 41.79411, 12.5118 41.79413, 12.51355 41.79421, 12.51369 41.79422, 12.51413 41.79425, 12.51563 41.79437, 12.51616 41.79442, 12.52077 41.7948, 12.52142 41.79486, 12.52244 41.79495, 12.52544 41.79526, 12.52803 41.79572, 12.52858 41.79584, 12.53114 41.79639, 12.53235 41.79666, 12.53419 41.79705, 12.53463 41.79715, 12.5356 41.79737, 12.53748 41.79778, 12.5377 41.79783, 12.5379 41.79787, 12.53806 41.79791, 12.53902 41.79812, 12.53985 41.79831, 12.54864 41.8002, 12.55144 41.80098, 12.55159 41.80103, 12.55502 41.80238, 12.55681 41.80329, 12.55706 41.80343, 12.55773 41.80378, 12.55896 41.80449, 12.55981 41.80495, 12.56118 41.80573, 12.56325 41.80688, 12.56817 41.80966, 12.56936 41.81032, 12.56972 41.81054, 12.5701 41.81075, 12.57037 41.8109, 12.57284 41.81236, 12.57289 41.81239, 12.57299 41.81245, 12.57437 41.81359, 12.57527 41.81465, 12.57563 41.81515, 12.57589 41.81556, 12.57626 41.81612, 12.57707 41.81731, 12.57715 41.81744, 12.57732 41.8177, 12.57811 41.81888, 12.57861 41.81964, 12.57888 41.82002, 12.57903 41.82026, 12.57928 41.82045, 12.57974 41.82093, 12.57977 41.82097, 12.58047 41.82182, 12.5806 41.822, 12.58065 41.82208, 12.58078 41.82229, 12.58094 41.82256, 12.581 41.82266, 12.58108 41.82281, 12.58133 41.82327, 12.58156 41.82378, 12.58226 41.82484, 12.58254 41.82528, 12.58302 41.82598, 12.58359 41.82687, 12.5843 41.82807, 12.58439 41.82821, 12.58454 41.82845, 12.58486 41.82898, 12.58564 41.83015, 12.5864 41.83125, 12.58676 41.83182, 12.58716 41.83241, 12.58731 41.83262, 12.58764 41.83306, 12.5877 41.83314, 12.58782 41.83326, 12.58824 41.83352, 12.58844 41.83375, 12.58879 41.83416, 12.58903 41.83468, 12.58943 41.83523, 12.58991 41.83555, 12.59065 41.83603, 12.59136 41.83621, 12.59173 41.83609, 12.59244 41.83561, 12.59303 41.83505, 12.5933 41.83477, 12.59348 41.83461, 12.59384 41.83424)","locationId":"c9e15a7d-b590-4720-827e-303a5b387b08","locationType":"PATH"},"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","thresholdsDefinition":{"thresholdsValues":{"warningThreshold":90.0,"criticalThreshold":100.0},"kpiThresholdsReference":"UNUSUAL"},"template":"EXPECTED_TRAVEL_TIME"...</t>
-  </si>
-  <si>
-    <t>Error: {"message":"You cannot perform the requested operation.","code":"AccessDenied","type":"Table","method":"deleteRowsAt","line":223}</t>
-  </si>
-  <si>
     <t xml:space="preserve">kpi name </t>
   </si>
   <si>
-    <t>2025-04-07T14:33:48.723Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:33:48.826Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:37:03.024Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:37:03.130Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:40:15.981Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:40:16.327Z</t>
-  </si>
-  <si>
-    <t>https://api.ptvgroup.tech/kpieng/v1/result/by-kpi-ids</t>
-  </si>
-  <si>
-    <t>Success: Retrieved length data for 34 KPIs</t>
-  </si>
-  <si>
-    <t>[{"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","timeStamp":"2025-04-07T14:32:00Z","results":[{"value":0.7160851,"defaultValue":0.67702585,"unusualValue":0.75992703,"averageValue":0.3549224,"progressive":1.2412142},{"value":0.113773584,"defaultValue":0.10963637,"unusualValue":0.12044343,"averageValue":0.05734928,"progressive":1.4422141},{"value":0.3090566,"defaultValue":0.29781818,"unusualValue":0.3090566,"averageValue":0.15452428,"progressive":1.9882141},{"value":0.06735849,"defaultValue":0.06490909,"unusualValue":0.06735849,"averageValue":0.033678368,"progressive":2.1072142},{"value":0.2609434,"defaultValue":0.21276924,"unusualValue":0.2609434,"averageValue":0.13046831,"progressive":2.5682142},{"value":0.14660378,"defaultValue":0.119538456,"unusualValue":0.14660378,"averageValue":0.07329998,"progressive":2.8272142},{"value":0.0356978,"defaultValue":0.029076923,"unusualValue":0.03566038,"averageValue":0.017829726,"progressive":2.8902142},{"value":0.15962264,"defaultValue":0.188,"unusualValue":0.15962264,"averageValue":0.07963559,"progressive":3.1722143},{"value":0.027169812,"defaultValue":0.032,"unusualValue":0.027169812,"averageValue":0.013540026,"progressive":3.2202144},{"value":0.20004307,"defaultValue":0.23533332,"unusualValue":0.19981131,"averageValue":0.0995756,"progressive":3.5732143},{"value":0.07209581,"defaultValue":0.085999995,"unusualValue":0.073018864,"averageValue":0.03638882,"progressive":3.7022142},{"value":0.016981132,"defaultValue":0.02,"unusualValue":0.016981132,"averageValue":0.008462516,"progressive":3.7322142},{"value":0.06905661,"defaultValue":0.08133334,"unusualValue":0.06905661,"averageValue":0.03441423,"progressive":3.8542142},{"value":0.03283019,"defaultValue":0.038666666,"unusualValue":0.03283019,"averageValue":0.016360864,"progressive":3.9122143},{"value":0.23046982,"defaultValue":0.26933336,"unusualValue":0.22867925,"averageValue":0.11396188,"progressive":4.316214},{"value":0.068490565,"defaultValue":0.08066667,"unusualValue":0.068490565,"averageValue":0.03416988,"progressive":4.437214},{"value":0.28740928,"defaultValue":0.33800003,"unusualValue":0.28698114,"averageValue":0.14301652,"progressive":4.944214},{"value":0.032236435,"defaultValue":0.02676923,"unusualValue":0.031926606,"averageValue":0.015931344,"progressive":5.002214},{"value":0.024770644,"defaultValue":0.020769231,"unusualValue":0.024770644,"averageValue":0.012367469,"progressive":5.047214},{"value":0.059999995,"defaultValue":0.05030769,"unusualValue":0.059999995,"averageValue":0.029939938,"progressive":5.156214},{"value":0.052844036,"defaultValue":0.044307694,"unusualValue":0.052844036,"averageValue":0.02636912,"progressive":5.2522144},{"value":0.01531915,"defaultValue":0.012923078,"unusualValue":0.015412845,"averageValue":0.007690994,"progressive":5.2802143},{"value":0.030275228,"defaultValue":0.025384614,"unusualValue":0.030275228,"averageValue":0.0151073085,"progressive":5.335214},{"value":0.0679797,"defaultValue":0.05723077,"unusualValue":0.068256885,"averageValue":0.034060117,"progressive":5.459214},{"value":0.005492958,"defaultValue":0.0046153846,"unusualValue":0.005504587,"averageValue":0.0027467834,"progressive":5.4692144},{"value":0.045137618,"defaultValue":0.037846155,"unusualValue":0.045137618,"averageValue":0.045072556,"progressive":5.551214},{"value":0.066836044,"defaultValue":0.056307696,"unusualValue":0.067155965,"averageValue":0.06702152,"progressive":5.6732144},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.009339064,"progressive":5.6902146},{"value":0.29669726,"defaultValue":0.24876921,"unusualValue":0.29669726,"averageValue":0.29610327,"progressive":6.2292147},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.009339064,"progressive":6.246215},{"value":0.18,"defaultValue":0.15092307,"unusualValue":0.18,"averageValue":0.17963965,"progressive":6.573215},{"value":0.0814679,"defaultValue":0.06830769,"unusualValue":0.0814679,"averageValue":0.081304796,"progressive":6.7212152},{"value":0.006055046,"defaultValue":0.005076923,"unusualValue":0.006055046,"averageValue":0.006042924,"progressive":6.7322154},{"value":0.080235526,"defaultValue":0.067384616,"unusualValue":0.08036697,"averageValue":0.080206074,"progressive":6.8782153},{"value":0.058348626,"defaultValue":0.048923075,"unusualValue":0.058348626,"averageValue":0.058231812,"progressive":6.9842153},{"value":0.20311926,"defaultValue":0.17030768,"unusualValue":0.20311926,"averageValue":0.20271263,"progressive":7.353215},{"value":0.0066055045,"defaultValue":0.0055384617,"unusualValue":0.0066055045,"averageValue":0.00659228,"progressive":7.3652153},{"value":0.04293578,"defaultValue":0.036000002,"unusualValue":0.04293578,"averageValue":0.042873893,"progressive":7.4432154},{"value":0.041553956,"defaultValue":0.035076924,"unusualValue":0.04183486,"averageValue":0.04175111,"progressive":7.5192156},{"value":0.3253211,"defaultValue":0.27276924,"unusualValue":0.3253211,"avera...</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:40:18.535Z</t>
-  </si>
-  <si>
-    <t>Success: Added 17 rows to KPI_list table</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:56:46.333Z</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:56:46.840Z</t>
-  </si>
-  <si>
-    <t>[{"kpiId":"d4377835-aa86-4873-93a8-a7936aff6dcd","timeStamp":"2025-04-07T14:47:00Z","results":[{"value":0.702574,"defaultValue":0.67702585,"unusualValue":0.702574,"averageValue":0.351287,"progressive":1.2412142},{"value":0.11940594,"defaultValue":0.10963637,"unusualValue":0.113773584,"averageValue":0.056886792,"progressive":1.4422141},{"value":0.3090566,"defaultValue":0.29781818,"unusualValue":0.3090566,"averageValue":0.1545283,"progressive":1.9882141},{"value":0.06735849,"defaultValue":0.06490909,"unusualValue":0.06735849,"averageValue":0.033679243,"progressive":2.1072142},{"value":0.2609434,"defaultValue":0.21276924,"unusualValue":0.2609434,"averageValue":0.1304717,"progressive":2.5682142},{"value":0.14660378,"defaultValue":0.119538456,"unusualValue":0.14660378,"averageValue":0.07330189,"progressive":2.8272142},{"value":0.03568966,"defaultValue":0.029076923,"unusualValue":0.03566038,"averageValue":0.01783019,"progressive":2.8902142},{"value":0.15962264,"defaultValue":0.188,"unusualValue":0.15962264,"averageValue":0.07981132,"progressive":3.1722143},{"value":0.027169812,"defaultValue":0.032,"unusualValue":0.027169812,"averageValue":0.013584906,"progressive":3.2202144},{"value":0.19998284,"defaultValue":0.23533332,"unusualValue":0.19981131,"averageValue":0.099905655,"progressive":3.5732143},{"value":0.073018864,"defaultValue":0.085999995,"unusualValue":0.073018864,"averageValue":0.036509432,"progressive":3.7022142},{"value":0.016981132,"defaultValue":0.02,"unusualValue":0.016981132,"averageValue":0.008490566,"progressive":3.7322142},{"value":0.06905661,"defaultValue":0.08133334,"unusualValue":0.06905661,"averageValue":0.034528304,"progressive":3.8542142},{"value":0.03283019,"defaultValue":0.038666666,"unusualValue":0.03283019,"averageValue":0.016415095,"progressive":3.9122143},{"value":0.23004995,"defaultValue":0.26933336,"unusualValue":0.22867925,"averageValue":0.11433963,"progressive":4.316214},{"value":0.0686322,"defaultValue":0.08066667,"unusualValue":0.068490565,"averageValue":0.034245282,"progressive":4.437214},{"value":0.28698114,"defaultValue":0.33800003,"unusualValue":0.28698114,"averageValue":0.14349057,"progressive":4.944214},{"value":0.031926606,"defaultValue":0.02676923,"unusualValue":0.031926606,"averageValue":0.015891396,"progressive":5.002214},{"value":0.024770644,"defaultValue":0.020769231,"unusualValue":0.024770644,"averageValue":0.01234193,"progressive":5.047214},{"value":0.059999995,"defaultValue":0.05030769,"unusualValue":0.059999995,"averageValue":0.029894892,"progressive":5.156214},{"value":0.052844036,"defaultValue":0.044307694,"unusualValue":0.052844036,"averageValue":0.026329448,"progressive":5.2522144},{"value":0.015412845,"defaultValue":0.012923078,"unusualValue":0.015412845,"averageValue":0.007679423,"progressive":5.2802143},{"value":0.030275228,"defaultValue":0.025384614,"unusualValue":0.030275228,"averageValue":0.01508458,"progressive":5.335214},{"value":0.068103425,"defaultValue":0.05723077,"unusualValue":0.068256885,"averageValue":0.03400887,"progressive":5.459214},{"value":0.005504587,"defaultValue":0.0046153846,"unusualValue":0.005504587,"averageValue":0.002742651,"progressive":5.4692144},{"value":0.045137618,"defaultValue":0.037846155,"unusualValue":0.045137618,"averageValue":0.044979475,"progressive":5.551214},{"value":0.067155965,"defaultValue":0.056307696,"unusualValue":0.067155965,"averageValue":0.06692068,"progressive":5.6732144},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.0093250135,"progressive":5.6902146},{"value":0.29669726,"defaultValue":0.24876921,"unusualValue":0.29669726,"averageValue":0.29565778,"progressive":6.2292147},{"value":0.009357799,"defaultValue":0.007846154,"unusualValue":0.009357799,"averageValue":0.0093250135,"progressive":6.246215},{"value":0.17806011,"defaultValue":0.15092307,"unusualValue":0.18,"averageValue":0.17936938,"progressive":6.573215},{"value":0.0814679,"defaultValue":0.06830769,"unusualValue":0.0814679,"averageValue":0.08118247,"progressive":6.7212152},{"value":0.006055046,"defaultValue":0.005076923,"unusualValue":0.006055046,"averageValue":0.0060338317,"progressive":6.7322154},{"value":0.08036697,"defaultValue":0.067384616,"unusualValue":0.08036697,"averageValue":0.080085404,"progressive":6.8782153},{"value":0.058348626,"defaultValue":0.048923075,"unusualValue":0.058348626,"averageValue":0.0581442,"progressive":6.9842153},{"value":0.20311926,"defaultValue":0.17030768,"unusualValue":0.20311926,"averageValue":0.20240763,"progressive":7.353215},{"value":0.0066055045,"defaultValue":0.0055384617,"unusualValue":0.0066055045,"averageValue":0.006582362,"progressive":7.3652153},{"value":0.04293578,"defaultValue":0.036000002,"unusualValue":0.04293578,"averageValue":0.042785354,"progressive":7.4432154},{"value":0.041517448,"defaultValue":0.035076924,"unusualValue":0.04183486,"averageValue":0.041688293,"progressive":7.5192156},{"value":0.3253211,"defaultValue":0.27276924,"unusualValue":0.3253211,"...</t>
-  </si>
-  <si>
-    <t>2025-04-07T14:56:48.968Z</t>
+    <t>fromTime (ISO 8601 format) UTC</t>
+  </si>
+  <si>
+    <t>toTime (ISO 8601 format) UTC</t>
+  </si>
+  <si>
+    <t>input date/time in your timezone accordingly with cell D5</t>
+  </si>
+  <si>
+    <t>Hour Difference with UTC  (0,+1,+2,-1,-2  etc)</t>
+  </si>
+  <si>
+    <t>UTC Time</t>
   </si>
   <si>
     <r>
@@ -339,6 +308,7 @@
     <r>
       <rPr>
         <b/>
+        <u/>
         <sz val="12"/>
         <color theme="5"/>
         <rFont val="Calibri"/>
@@ -350,6 +320,7 @@
     <r>
       <rPr>
         <b/>
+        <u/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
@@ -360,24 +331,19 @@
     </r>
   </si>
   <si>
-    <t>apiKey</t>
-  </si>
-  <si>
-    <t>fromTime (ISO 8601 format) UTC</t>
-  </si>
-  <si>
-    <t>toTime (ISO 8601 format) UTC</t>
+    <t>your api key</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm\ \ \(\U\T\C\)"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,14 +377,6 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="5"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -467,8 +425,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -495,6 +477,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -611,19 +599,19 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -641,11 +629,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
@@ -653,10 +641,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -673,26 +657,23 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -708,6 +689,27 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -715,6 +717,42 @@
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="21">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <font>
         <sz val="11"/>
@@ -746,26 +784,6 @@
       </font>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -779,22 +797,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="15" formatCode="0.00E+00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -3017,25 +3019,25 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F22" insertRow="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="18">
   <autoFilter ref="A20:F21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="16" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="15" totalsRowDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="14" totalsRowDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="13" totalsRowDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="12" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}" name="RequestLog" displayName="RequestLog" ref="A1:D12" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:D12" xr:uid="{AC3C69C9-D4DE-4DBF-B52D-21EAB47C1AF4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{12C99960-E3F9-43EE-AB30-77013461C383}" name="RequestLog" displayName="RequestLog" ref="A1:D2" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:D2" xr:uid="{12C99960-E3F9-43EE-AB30-77013461C383}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{94788DBD-DB73-4499-9554-13FD83D56E99}" name="Datetime" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{1B49E132-7BC4-47FA-B194-A8662469036D}" name="Request URL" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{EFFC061F-6CE6-47DD-B6F4-8B601FE36300}" name="Status" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{8A164B4F-6F22-4123-A5F9-CE61462B18B6}" name="Body (answer)" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{4F756C8E-2C1D-4929-8AA2-36FBE76BB654}" name="Datetime" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{F510F3D1-4460-4F54-8E2B-AC1ADD028DAD}" name="Request URL" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{1E35CCD3-4AB8-44AB-8BB9-97B0A53C61E4}" name="Status" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{8ADA9E94-3D8C-4423-8126-112691360514}" name="Body (answer)" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3305,10 +3307,33 @@
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B5" dT="2025-04-07T15:11:20.63" personId="{FE2F6ED8-9348-4908-88B0-71F732C27369}" id="{248F8340-0CF6-49E4-A52E-0AEFCE99FCE3}">
-    <text>Attention, Time and Date in UTC</text>
+    <text xml:space="preserve">Attention, Time and Date in your timezone including DST for doubts go to Time Difference between UTC, Time Zone and the World </text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1804882917</xltc2:checksum>
+        <xltc2:hyperlink startIndex="73" length="52" url="https://www.timeanddate.com/time/difference/timezone/utc"/>
+      </x:ext>
+    </extLst>
   </threadedComment>
   <threadedComment ref="C5" dT="2025-04-07T15:11:28.96" personId="{FE2F6ED8-9348-4908-88B0-71F732C27369}" id="{B6F9E66B-90DE-4A4B-B43D-3E8DA64FE905}">
-    <text>Attention, Time and Date in UTC</text>
+    <text xml:space="preserve">Attention, Time and Date in your timezone including DST for doubts go to Time Difference between UTC, Time Zone and the World 
+</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1406914764</xltc2:checksum>
+        <xltc2:hyperlink startIndex="73" length="52" url="https://www.timeanddate.com/time/difference/timezone/utc"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="D5" dT="2025-04-08T15:22:15.18" personId="{FE2F6ED8-9348-4908-88B0-71F732C27369}" id="{716D20F0-8F3A-44D5-9F55-DB8295C640BA}">
+    <text xml:space="preserve">Delta in hours between your timezone including current DST if active and the UTC time, in case of doubts go to  to Time Difference between UTC, Time Zone and the World 
+</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>1796391628</xltc2:checksum>
+        <xltc2:hyperlink startIndex="115" length="52" url="https://www.timeanddate.com/time/difference/timezone/utc"/>
+      </x:ext>
+    </extLst>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -3340,7 +3365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G296"/>
+  <dimension ref="A1:I313"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
@@ -3355,30 +3380,32 @@
     <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8"/>
+      <c r="D1" s="33" t="s">
+        <v>52</v>
+      </c>
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
     </row>
-    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>3</v>
@@ -3386,16 +3413,19 @@
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I2" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="22" t="str">
+        <v>46</v>
+      </c>
+      <c r="B3" s="21" t="str">
         <f>TEXT(B4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B5, "HH:MM:SS") &amp; "Z"</f>
         <v>2025-03-01T00:00:00Z</v>
       </c>
-      <c r="C3" s="23" t="str">
+      <c r="C3" s="22" t="str">
         <f>TEXT(C4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C5, "HH:MM:SS") &amp; "Z"</f>
         <v>2025-03-01T23:59:00Z</v>
       </c>
@@ -3407,10 +3437,13 @@
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
-    </row>
-    <row r="4" spans="1:7" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>66</v>
+      <c r="I3" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="29" t="s">
+        <v>49</v>
       </c>
       <c r="B4" s="14">
         <v>45717</v>
@@ -3418,82 +3451,90 @@
       <c r="C4" s="14">
         <v>45717</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>4</v>
+      <c r="D4" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
-    </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="16">
+      <c r="I4" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="15">
         <v>0</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="15">
         <v>0.99930555555555556</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>7</v>
+      <c r="D5" s="28">
+        <v>2</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8" t="s">
-        <v>8</v>
+      <c r="I5" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="30">
+        <f>B4+B5-TIME($D$5,0,0)</f>
+        <v>45716.916666666664</v>
+      </c>
+      <c r="C6" s="31">
+        <f>C4+C5-TIME($D$5,0,0)</f>
+        <v>45717.915972222218</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>51</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I6" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
-      <c r="D7" s="8" t="s">
-        <v>9</v>
-      </c>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
-      <c r="D8" s="8" t="s">
-        <v>10</v>
-      </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
-      <c r="E9" s="17"/>
+      <c r="E9" s="16"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
-      <c r="E10" s="18"/>
+      <c r="E10" s="17"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
     </row>
-    <row r="11" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -3502,7 +3543,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -3511,7 +3552,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -3520,7 +3561,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -3529,7 +3570,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -3538,7 +3579,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -3552,20 +3593,20 @@
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="28"/>
-      <c r="G17" s="29"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="27"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
@@ -3598,388 +3639,456 @@
       <c r="G20" s="8"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="19"/>
+      <c r="A21" s="18"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="21"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
+      <c r="A22" s="18"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
-      <c r="F22" s="24"/>
+      <c r="F22" s="35"/>
       <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
+      <c r="A23" s="18"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
       <c r="E23" s="8"/>
-      <c r="F23" s="20"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="8"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="19"/>
+      <c r="A24" s="18"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
-      <c r="F24" s="20"/>
+      <c r="F24" s="19"/>
       <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="19"/>
+      <c r="A25" s="18"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
-      <c r="F25" s="20"/>
+      <c r="F25" s="19"/>
       <c r="G25" s="8"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="19"/>
+      <c r="A26" s="18"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
       <c r="E26" s="8"/>
-      <c r="F26" s="20"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
+      <c r="A27" s="18"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
-      <c r="F27" s="20"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="8"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="19"/>
+      <c r="A28" s="18"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
-      <c r="F28" s="20"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="8"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="19"/>
+      <c r="A29" s="18"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
-      <c r="F29" s="20"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="8"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="19"/>
+      <c r="A30" s="18"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
       <c r="D30" s="8"/>
       <c r="E30" s="8"/>
-      <c r="F30" s="20"/>
+      <c r="F30" s="19"/>
       <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="19"/>
+      <c r="A31" s="18"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
-      <c r="F31" s="20"/>
+      <c r="F31" s="19"/>
       <c r="G31" s="8"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="19"/>
+      <c r="A32" s="18"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
-      <c r="F32" s="20"/>
+      <c r="F32" s="19"/>
       <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="19"/>
+      <c r="A33" s="18"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
-      <c r="F33" s="20"/>
+      <c r="F33" s="19"/>
       <c r="G33" s="8"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="19"/>
+      <c r="A34" s="18"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
       <c r="E34" s="8"/>
-      <c r="F34" s="20"/>
+      <c r="F34" s="19"/>
       <c r="G34" s="8"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="19"/>
+      <c r="A35" s="18"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
-      <c r="F35" s="20"/>
+      <c r="F35" s="19"/>
       <c r="G35" s="8"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="19"/>
+      <c r="A36" s="18"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
-      <c r="F36" s="20"/>
+      <c r="F36" s="19"/>
       <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="19"/>
+      <c r="A37" s="18"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
-      <c r="F37" s="20"/>
+      <c r="F37" s="19"/>
       <c r="G37" s="8"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="19"/>
+      <c r="A38" s="18"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
-      <c r="F38" s="20"/>
+      <c r="F38" s="19"/>
       <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="19"/>
+      <c r="A39" s="18"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
-      <c r="F39" s="20"/>
+      <c r="F39" s="19"/>
       <c r="G39" s="8"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="19"/>
+      <c r="A40" s="18"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
       <c r="E40" s="8"/>
-      <c r="F40" s="20"/>
+      <c r="F40" s="19"/>
       <c r="G40" s="8"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="19"/>
+      <c r="A41" s="18"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
       <c r="E41" s="8"/>
-      <c r="F41" s="20"/>
+      <c r="F41" s="19"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="19"/>
+      <c r="A42" s="18"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
       <c r="E42" s="8"/>
-      <c r="F42" s="20"/>
+      <c r="F42" s="19"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="19"/>
+      <c r="A43" s="18"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
-      <c r="F43" s="20"/>
+      <c r="F43" s="19"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="19"/>
+      <c r="A44" s="18"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
-      <c r="F44" s="20"/>
+      <c r="F44" s="19"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="19"/>
+      <c r="A45" s="18"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
-      <c r="F45" s="20"/>
+      <c r="F45" s="19"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="19"/>
+      <c r="A46" s="18"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
       <c r="E46" s="8"/>
-      <c r="F46" s="20"/>
+      <c r="F46" s="19"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="19"/>
+      <c r="A47" s="18"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
       <c r="D47" s="8"/>
       <c r="E47" s="8"/>
-      <c r="F47" s="20"/>
+      <c r="F47" s="19"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="19"/>
+      <c r="A48" s="18"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
-      <c r="F48" s="20"/>
+      <c r="F48" s="19"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="19"/>
+      <c r="A49" s="18"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
-      <c r="F49" s="20"/>
+      <c r="F49" s="19"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="19"/>
+      <c r="A50" s="18"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
-      <c r="F50" s="20"/>
+      <c r="F50" s="19"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="19"/>
+      <c r="A51" s="18"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
       <c r="D51" s="8"/>
       <c r="E51" s="8"/>
-      <c r="F51" s="20"/>
+      <c r="F51" s="19"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="19"/>
+      <c r="A52" s="18"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
       <c r="D52" s="8"/>
       <c r="E52" s="8"/>
-      <c r="F52" s="20"/>
+      <c r="F52" s="19"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="19"/>
+      <c r="A53" s="18"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
-      <c r="F53" s="20"/>
+      <c r="F53" s="19"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="19"/>
+      <c r="A54" s="18"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
-      <c r="F54" s="20"/>
+      <c r="F54" s="19"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="19"/>
+      <c r="A55" s="18"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
-      <c r="F55" s="20"/>
+      <c r="F55" s="19"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="8"/>
+      <c r="A56" s="18"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
-      <c r="F56" s="20"/>
+      <c r="F56" s="19"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="19"/>
+      <c r="A57" s="18"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
       <c r="E57" s="8"/>
-      <c r="F57" s="20"/>
+      <c r="F57" s="19"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="1"/>
-      <c r="F58" s="4"/>
+      <c r="A58" s="18"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="19"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-      <c r="F59" s="4"/>
+      <c r="A59" s="18"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="19"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-      <c r="F60" s="4"/>
+      <c r="A60" s="18"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="19"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="1"/>
-      <c r="F61" s="4"/>
+      <c r="A61" s="18"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="8"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="19"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="1"/>
-      <c r="F62" s="4"/>
+      <c r="A62" s="18"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="19"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="1"/>
-      <c r="F63" s="4"/>
+      <c r="A63" s="18"/>
+      <c r="B63" s="8"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="19"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="1"/>
-      <c r="F64" s="4"/>
+      <c r="A64" s="18"/>
+      <c r="B64" s="8"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="19"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="1"/>
-      <c r="F65" s="4"/>
+      <c r="A65" s="18"/>
+      <c r="B65" s="8"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="19"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="1"/>
-      <c r="F66" s="4"/>
+      <c r="A66" s="18"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="19"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="1"/>
-      <c r="F67" s="4"/>
+      <c r="A67" s="18"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="19"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="1"/>
-      <c r="F68" s="4"/>
+      <c r="A68" s="18"/>
+      <c r="B68" s="8"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="19"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="1"/>
-      <c r="F69" s="4"/>
+      <c r="A69" s="18"/>
+      <c r="B69" s="8"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="8"/>
+      <c r="F69" s="19"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="1"/>
-      <c r="F70" s="4"/>
+      <c r="A70" s="18"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="19"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="1"/>
-      <c r="F71" s="4"/>
+      <c r="A71" s="18"/>
+      <c r="B71" s="8"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="8"/>
+      <c r="E71" s="8"/>
+      <c r="F71" s="19"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="1"/>
-      <c r="F72" s="4"/>
+      <c r="A72" s="18"/>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="19"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="1"/>
-      <c r="F73" s="4"/>
+      <c r="A73" s="8"/>
+      <c r="B73" s="8"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="8"/>
+      <c r="E73" s="8"/>
+      <c r="F73" s="19"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="1"/>
-      <c r="F74" s="4"/>
+      <c r="A74" s="18"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="8"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="19"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
@@ -4198,24 +4307,31 @@
       <c r="F128" s="4"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" s="1"/>
       <c r="F129" s="4"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" s="1"/>
       <c r="F130" s="4"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="1"/>
       <c r="F131" s="4"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" s="1"/>
       <c r="F132" s="4"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="1"/>
       <c r="F133" s="4"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="1"/>
       <c r="F134" s="4"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="1"/>
       <c r="F135" s="4"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -4259,31 +4375,24 @@
       <c r="F145" s="4"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A146" s="1"/>
       <c r="F146" s="4"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A147" s="1"/>
       <c r="F147" s="4"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A148" s="1"/>
       <c r="F148" s="4"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A149" s="1"/>
       <c r="F149" s="4"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A150" s="1"/>
       <c r="F150" s="4"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A151" s="1"/>
       <c r="F151" s="4"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A152" s="1"/>
       <c r="F152" s="4"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -4364,51 +4473,67 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="1"/>
+      <c r="F172" s="4"/>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="1"/>
+      <c r="F173" s="4"/>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="1"/>
+      <c r="F174" s="4"/>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="1"/>
+      <c r="F175" s="4"/>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="1"/>
+      <c r="F176" s="4"/>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="1"/>
+      <c r="F177" s="4"/>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="1"/>
+      <c r="F178" s="4"/>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="1"/>
+      <c r="F179" s="4"/>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="1"/>
+      <c r="F180" s="4"/>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="1"/>
+      <c r="F181" s="4"/>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
+      <c r="F182" s="4"/>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
+      <c r="F183" s="4"/>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
+      <c r="F184" s="4"/>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
+      <c r="F185" s="4"/>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
+      <c r="F186" s="4"/>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
+      <c r="F187" s="4"/>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
@@ -4416,98 +4541,120 @@
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
-      <c r="F189" s="4"/>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
-      <c r="F190" s="4"/>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
-      <c r="F191" s="4"/>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
-      <c r="F192" s="4"/>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
-      <c r="F193" s="4"/>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
-      <c r="F194" s="4"/>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
-      <c r="F195" s="4"/>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F196" s="4"/>
+      <c r="A196" s="1"/>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F197" s="4"/>
+      <c r="A197" s="1"/>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F198" s="4"/>
+      <c r="A198" s="1"/>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F199" s="4"/>
+      <c r="A199" s="1"/>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F200" s="4"/>
+      <c r="A200" s="1"/>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F201" s="4"/>
+      <c r="A201" s="1"/>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F202" s="4"/>
+      <c r="A202" s="1"/>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
-      <c r="F203" s="4"/>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
-      <c r="F204" s="4"/>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
+      <c r="F205" s="4"/>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
+      <c r="F206" s="4"/>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
+      <c r="F207" s="4"/>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
-    </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F208" s="4"/>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
-    </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F209" s="4"/>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" s="1"/>
-    </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F210" s="4"/>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" s="1"/>
-    </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A219" s="1"/>
-    </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F211" s="4"/>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A212" s="1"/>
+      <c r="F212" s="4"/>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F213" s="4"/>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F214" s="4"/>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F215" s="4"/>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F216" s="4"/>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F217" s="4"/>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F218" s="4"/>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F219" s="4"/>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" s="1"/>
-    </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F220" s="4"/>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="1"/>
-    </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="F221" s="4"/>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" s="1"/>
     </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" s="1"/>
     </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" s="1"/>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.25">
@@ -4519,20 +4666,50 @@
     <row r="227" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A227" s="1"/>
     </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228" s="1"/>
+    </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A236" s="1"/>
     </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A252" s="1"/>
-    </row>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A268" s="1"/>
-    </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A295" s="1"/>
-    </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A296" s="1"/>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237" s="1"/>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238" s="1"/>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239" s="1"/>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240" s="1"/>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" s="1"/>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" s="1"/>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" s="1"/>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" s="1"/>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" s="1"/>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" s="1"/>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" s="1"/>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312" s="1"/>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313" s="1"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
@@ -4540,7 +4717,7 @@
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E17:G17"/>
   </mergeCells>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <dataValidations count="4">
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a correct date" error="please input a correct date_x000a_" sqref="B4:C4" xr:uid="{F83F3375-2F4B-4A5A-9230-C8D6497346A1}">
       <formula1>45658</formula1>
@@ -4551,10 +4728,11 @@
       <formula2>0.999305555555556</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3" xr:uid="{9367E08E-DE83-4A16-AE23-738728604C7E}">
-      <formula1>$D$4:$D$8</formula1>
+      <formula1>$I$2:$I$6</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:C3" xr:uid="{5AD50032-6A28-44BB-BCD8-0C40654E1CEC}">
-      <formula1>AND(ISNUMBER(FIND("T", A1)), ISNUMBER(FIND("Z", A1)), LEN(A1)=20, ISNUMBER(DATEVALUE(LEFT(A1, 10))), ISNUMBER(TIMEVALUE(MID(A1, 12, 8))))</formula1>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5" xr:uid="{7150081A-FE65-4EDE-A8F0-5F7D4D5D7E40}">
+      <formula1>-12</formula1>
+      <formula2>12</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4569,7 +4747,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -4579,146 +4757,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="34" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>62</v>
-      </c>
-      <c r="B10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" t="s">
-        <v>61</v>
-      </c>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="34"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4863,28 +4919,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
-</scriptIds>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -5113,6 +5147,28 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
+</scriptIds>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5125,23 +5181,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5160,6 +5199,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
timezone now works also with negative value and has a button to helo tp get the right timezone
timezone now works also with negative value and has a button to helo tp get the right timezone
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="551" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{094FED43-8375-4948-BC31-A585458D2D51}"/>
+  <xr:revisionPtr revIDLastSave="580" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EC3B46E-259E-4C15-BF59-42A53EA12099}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -343,7 +343,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm\ \ \(\U\T\C\)"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,19 +417,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -601,7 +588,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -666,8 +653,16 @@
     <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -689,25 +684,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -717,42 +694,6 @@
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="21">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="15" formatCode="0.00E+00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
     <dxf>
       <font>
         <sz val="11"/>
@@ -784,6 +725,26 @@
       </font>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -797,6 +758,22 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="15" formatCode="0.00E+00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -3006,6 +2983,90 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>200025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1838325</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Rectangle: Rounded Corners 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C4AC8B6B-5928-403D-9018-DF6CF89C747F}"/>
+            </a:ext>
+            <a:ext uri="{6ECC49D1-AA05-4338-93AA-15A1B29DFB0A}">
+              <asl:scriptLink xmlns:asl="http://schemas.microsoft.com/office/drawing/2021/scriptlink" val="{&quot;shareId&quot;:&quot;ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VkcGJtb18yQlBOTXFlb0RheDh0eTB3QnNZeHJGOHA1dnF4TEhWUFpKWnRDMXc&quot;}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8772525" y="1924050"/>
+          <a:ext cx="2247900" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>Get Delta</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" baseline="0"/>
+            <a:t> of your time versus UTC</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-150"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3019,25 +3080,25 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}" name="KPI_list" displayName="KPI_list" ref="A20:F22" insertRow="1" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" totalsRowDxfId="18">
   <autoFilter ref="A20:F21" xr:uid="{E4C48AEB-FCAF-42A7-BECC-DCC22D55EF4F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="16" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="15" totalsRowDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="14" totalsRowDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="13" totalsRowDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="12" totalsRowDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{56E38A3E-FD68-4D89-84C5-32CCE3CA1ED3}" name="KPI ID" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{F16CC454-78F1-40FA-90CE-7ABD5E207C06}" name="KPI Name" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{B8989DFD-A2D5-46DB-8DC4-D1C516A8A673}" name="Location Name" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{C69B7F3F-008E-4546-87DB-1B3DC783425F}" name="Location ID" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{C986407E-E482-405A-9426-89C162FF4F04}" name="Km Length" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{D4015B30-F19B-4377-9B88-6668F60F09C8}" name="KPI url" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{12C99960-E3F9-43EE-AB30-77013461C383}" name="RequestLog" displayName="RequestLog" ref="A1:D2" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{12C99960-E3F9-43EE-AB30-77013461C383}" name="RequestLog" displayName="RequestLog" ref="A1:D2" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A1:D2" xr:uid="{12C99960-E3F9-43EE-AB30-77013461C383}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4F756C8E-2C1D-4929-8AA2-36FBE76BB654}" name="Datetime" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{F510F3D1-4460-4F54-8E2B-AC1ADD028DAD}" name="Request URL" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{1E35CCD3-4AB8-44AB-8BB9-97B0A53C61E4}" name="Status" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{8ADA9E94-3D8C-4423-8126-112691360514}" name="Body (answer)" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{4F756C8E-2C1D-4929-8AA2-36FBE76BB654}" name="Datetime" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{F510F3D1-4460-4F54-8E2B-AC1ADD028DAD}" name="Request URL" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1E35CCD3-4AB8-44AB-8BB9-97B0A53C61E4}" name="Status" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{8ADA9E94-3D8C-4423-8126-112691360514}" name="Body (answer)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3390,7 +3451,7 @@
       <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="24" t="s">
         <v>52</v>
       </c>
       <c r="E1" s="8"/>
@@ -3422,12 +3483,12 @@
         <v>46</v>
       </c>
       <c r="B3" s="21" t="str">
-        <f>TEXT(B4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B5, "HH:MM:SS") &amp; "Z"</f>
-        <v>2025-03-01T00:00:00Z</v>
-      </c>
-      <c r="C3" s="22" t="str">
-        <f>TEXT(C4, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C5, "HH:MM:SS") &amp; "Z"</f>
-        <v>2025-03-01T23:59:00Z</v>
+        <f>TEXT(B6, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B6, "HH:MM:SS") &amp; "Z"</f>
+        <v>2025-02-28T22:00:00Z</v>
+      </c>
+      <c r="C3" s="21" t="str">
+        <f>TEXT(C6, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C6, "HH:MM:SS") &amp; "Z"</f>
+        <v>2025-03-01T21:59:00Z</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>4</v>
@@ -3442,7 +3503,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="23" t="s">
         <v>49</v>
       </c>
       <c r="B4" s="14">
@@ -3468,7 +3529,7 @@
       <c r="C5" s="15">
         <v>0.99930555555555556</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="22">
         <v>2</v>
       </c>
       <c r="E5" s="8"/>
@@ -3482,15 +3543,15 @@
       <c r="A6" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="30">
-        <f>B4+B5-TIME($D$5,0,0)</f>
+      <c r="B6" s="31">
+        <f>IF($D$5&gt;0,B4+B5-TIME($D$5,0,0),B4+B5+TIME(-1*$D$5,0,0))</f>
         <v>45716.916666666664</v>
       </c>
       <c r="C6" s="31">
-        <f>C4+C5-TIME($D$5,0,0)</f>
+        <f>IF($D$5&gt;0,C4+C5-TIME($D$5,0,0),C4+C5+TIME(-1*$D$5,0,0))</f>
         <v>45717.915972222218</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="31" t="s">
         <v>51</v>
       </c>
       <c r="E6" s="8"/>
@@ -3593,20 +3654,20 @@
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="26"/>
-      <c r="G17" s="27"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="30"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
@@ -3653,7 +3714,7 @@
       <c r="C22" s="8"/>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
-      <c r="F22" s="35"/>
+      <c r="F22" s="25"/>
       <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -4747,7 +4808,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C613D63-BEFF-438B-8428-B01B6B672385}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -4757,24 +4818,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4919,6 +4974,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -5147,29 +5211,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
-</scriptIds>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6">
@@ -5180,7 +5222,29 @@
 </p:properties>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP62LONI75QE6NGKT2QDNMPS3S2M:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VkcGJtb18yQlBOTXFlb0RheDh0eTB3QnNZeHJGOHA1dnF4TEhWUFpKWnRDMXc"/>
+</scriptIds>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5199,24 +5263,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5225,4 +5272,13 @@
     <ds:schemaRef ds:uri="43744f66-d8c7-4420-ad58-b4d72814d14f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fixed locale dependency  in date time settings
fixed local in date time settings
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptvgroup-my.sharepoint.com/personal/luca_paone_ptvgroup_com/Documents/Documents/GitHub/PTV-Mobility/PTV-Flows-tutorials/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luca.paone\github\PTV-Flows-tutorials\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="608" documentId="8_{0D0DBBFD-439C-4D97-BF73-A8B79CE62064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10DFCA55-887D-4264-9F77-3B89FD0E6538}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAB72E2-4BCD-4539-B0DD-61B8C3B7C266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -269,9 +269,6 @@
     <t>Hour Difference with UTC  (0,+1,+2,-1,-2  etc)</t>
   </si>
   <si>
-    <t>UTC Time</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">IN </t>
     </r>
@@ -340,15 +337,19 @@
   <si>
     <t>For the "Get HDA KPI DETAILED data" button, the time interval between From and To must not exceed 24 hours.</t>
   </si>
+  <si>
+    <t>yyyy-mm-dd UTC Time</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-150,1]hh:mm;@"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ hh:mm\ \ \(\U\T\C\)"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm\ \ \(\U\T\C\)"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -596,7 +597,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -674,6 +675,7 @@
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -694,7 +696,14 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -3075,6 +3084,175 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2362200</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>133349</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="361950" cy="332003"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="TextBox 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43941F79-AD55-4F62-9A96-A454B9D1F36F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2362200" y="2238374"/>
+          <a:ext cx="361950" cy="332003"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst>
+            <a:gd name="connsiteX0" fmla="*/ 0 w 361950"/>
+            <a:gd name="connsiteY0" fmla="*/ 166002 h 332003"/>
+            <a:gd name="connsiteX1" fmla="*/ 180975 w 361950"/>
+            <a:gd name="connsiteY1" fmla="*/ 0 h 332003"/>
+            <a:gd name="connsiteX2" fmla="*/ 361950 w 361950"/>
+            <a:gd name="connsiteY2" fmla="*/ 166002 h 332003"/>
+            <a:gd name="connsiteX3" fmla="*/ 180975 w 361950"/>
+            <a:gd name="connsiteY3" fmla="*/ 332004 h 332003"/>
+            <a:gd name="connsiteX4" fmla="*/ 0 w 361950"/>
+            <a:gd name="connsiteY4" fmla="*/ 166002 h 332003"/>
+          </a:gdLst>
+          <a:ahLst/>
+          <a:cxnLst>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX0" y="connsiteY0"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX1" y="connsiteY1"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX2" y="connsiteY2"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX3" y="connsiteY3"/>
+            </a:cxn>
+            <a:cxn ang="0">
+              <a:pos x="connsiteX4" y="connsiteY4"/>
+            </a:cxn>
+          </a:cxnLst>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="361950" h="332003" fill="none" extrusionOk="0">
+              <a:moveTo>
+                <a:pt x="0" y="166002"/>
+              </a:moveTo>
+              <a:cubicBezTo>
+                <a:pt x="1427" y="72966"/>
+                <a:pt x="82774" y="115"/>
+                <a:pt x="180975" y="0"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="287560" y="11341"/>
+                <a:pt x="344182" y="73940"/>
+                <a:pt x="361950" y="166002"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="376229" y="259753"/>
+                <a:pt x="273137" y="328450"/>
+                <a:pt x="180975" y="332004"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="66032" y="336478"/>
+                <a:pt x="3137" y="253430"/>
+                <a:pt x="0" y="166002"/>
+              </a:cubicBezTo>
+              <a:close/>
+            </a:path>
+            <a:path w="361950" h="332003" stroke="0" extrusionOk="0">
+              <a:moveTo>
+                <a:pt x="0" y="166002"/>
+              </a:moveTo>
+              <a:cubicBezTo>
+                <a:pt x="-9449" y="90900"/>
+                <a:pt x="67905" y="-5418"/>
+                <a:pt x="180975" y="0"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="288254" y="-1082"/>
+                <a:pt x="359353" y="79052"/>
+                <a:pt x="361950" y="166002"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="350554" y="261491"/>
+                <a:pt x="268488" y="346711"/>
+                <a:pt x="180975" y="332004"/>
+              </a:cubicBezTo>
+              <a:cubicBezTo>
+                <a:pt x="95103" y="322894"/>
+                <a:pt x="-16644" y="261500"/>
+                <a:pt x="0" y="166002"/>
+              </a:cubicBezTo>
+              <a:close/>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:ln w="57150">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:extLst>
+            <a:ext uri="{C807C97D-BFC1-408E-A445-0C87EB9F89A2}">
+              <ask:lineSketchStyleProps xmlns:ask="http://schemas.microsoft.com/office/drawing/2018/sketchyshapes" sd="981765707">
+                <a:prstGeom prst="ellipse">
+                  <a:avLst/>
+                </a:prstGeom>
+                <ask:type>
+                  <ask:lineSketchCurved/>
+                </ask:type>
+              </ask:lineSketchStyleProps>
+            </a:ext>
+          </a:extLst>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="lt1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>2</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-150" sz="1100" b="1">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3454,13 +3632,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
@@ -3491,12 +3669,12 @@
         <v>36</v>
       </c>
       <c r="B3" s="20" t="str">
-        <f>TEXT(B6, "YYYY-MM-DD") &amp; "T" &amp; TEXT(B6, "HH:MM:SS") &amp; "Z"</f>
-        <v>2025-02-28T22:00:00Z</v>
+        <f>YEAR(B6)&amp;"-"&amp;TEXT(MONTH(B6),"00")&amp;"-"&amp;TEXT(DAY(B6),"00")&amp;"T"&amp;TEXT(HOUR(B6),"00")&amp;":"&amp;TEXT(MINUTE(B6),"00")&amp;"Z"</f>
+        <v>2025-02-28T22:00Z</v>
       </c>
       <c r="C3" s="20" t="str">
-        <f>TEXT(C6, "YYYY-MM-DD") &amp; "T" &amp; TEXT(C6, "HH:MM:SS") &amp; "Z"</f>
-        <v>2025-03-01T21:59:00Z</v>
+        <f>YEAR(C6)&amp;"-"&amp;TEXT(MONTH(C6),"00")&amp;"-"&amp;TEXT(DAY(C6),"00")&amp;"T"&amp;TEXT(HOUR(C6),"00")&amp;":"&amp;TEXT(MINUTE(C6),"00")&amp;"Z"</f>
+        <v>2025-03-01T21:59Z</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>4</v>
@@ -3551,16 +3729,16 @@
       <c r="A6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="32">
         <f>IF($D$5&gt;0,B4+B5-TIME($D$5,0,0),B4+B5+TIME(-1*$D$5,0,0))</f>
         <v>45716.916666666664</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="32">
         <f>IF($D$5&gt;0,C4+C5-TIME($D$5,0,0),C4+C5+TIME(-1*$D$5,0,0))</f>
         <v>45717.915972222218</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -3571,8 +3749,8 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -3611,6 +3789,7 @@
       <c r="E11" s="12"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
+      <c r="I11" s="33"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
@@ -3662,20 +3841,20 @@
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="29"/>
-      <c r="G17" s="30"/>
+      <c r="E17" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="30"/>
+      <c r="G17" s="31"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
@@ -4855,12 +5034,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -4890,12 +5069,12 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
@@ -4904,8 +5083,8 @@
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="31" t="s">
-        <v>51</v>
+      <c r="A15" s="26" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -4953,7 +5132,7 @@
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -4963,7 +5142,7 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -4983,6 +5162,29 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP62LONI75QE6NGKT2QDNMPS3S2M:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VkcGJtb18yQlBOTXFlb0RheDh0eTB3QnNZeHJGOHA1dnF4TEhWUFpKWnRDMXc"/>
+</scriptIds>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002632A3CB0C6CDD4EA758E3E5A84892AF" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6c6c7bcb5e773f9f7da0ee88a749e050">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6" xmlns:ns3="43744f66-d8c7-4420-ad58-b4d72814d14f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ebd9547eaff2c58e2be891023bba85c" ns2:_="" ns3:_="">
     <xsd:import namespace="38e0ca72-0591-4ce1-b0f5-bc9dbb7a40b6"/>
@@ -5211,29 +5413,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP34CPJAWFB2KNH3KFLDAT7S6ZD5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYd1QwZ3NVT2xOUHRSVmpCUDh2WkgwQkVZczdTR3Z3ajNhejYxNDE0V2hubVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP35PIBPL3DEO5HKPJLU5P36S2CF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYMTZBdlhzWkhkT3A2VjA2X2ZwYUVVQjZiaGQ5cGVoTzQtNkhTM0c4blB4eUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZY6RAZF6AYIVH3DIVYMJWABBVA:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VUajBRWkw0R0VWUHNhSzRZbXdBaHFBQnY1c1lGTTlQOEZFek45N040eGJLUVE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP2KVIUFHFEDZVAL5VMMJDQOE2MB:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VVcXFLRk9VZzgxQXZ0V01TT0RpYVlFQjI0Zkg3a3hDU1dqWFBWcC13WG1Ba3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3TELXFVPETVFA3H5FVV4IEC6JU:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VYTWk3bHE4azZsQnNfUzFyeEJCZVRRQmhZZ19mcURpZkhTNkxCcGRyM3EyS3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP54UGBJU5OTTZCZF6HJETF77AOF:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VieWhncHAxMDU1Rmt2anBKTXZfZ2NVQmE1NU12TGdRRldDelA1ei1nU1VTd3c"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP3C4BP3UZJGJZHLSUIRS7NMP5RO:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VXTGdYN3BsSms1T3VWRVJsOXJIOWk0QlY2VmdJQk1oc1FOZTh5YTUtU1R5Vmc"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOPZMDL5LKT3J6VGJ3NYPAX6OFD2N:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VTd2EtclZQYWZWTW5iY1BCZnppajAwQnZ2Zmp5LWV6elRFTE5fQVpMa0RoUUE"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01WXRLOP62LONI75QE6NGKT2QDNMPS3S2M:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9wdHZncm91cC1teS5zaGFyZXBvaW50LmNvbS86dTovcC9sdWNhX3Bhb25lL0VkcGJtb18yQlBOTXFlb0RheDh0eTB3QnNZeHJGOHA1dnF4TEhWUFpKWnRDMXc"/>
-</scriptIds>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A45759AB-7D2D-4B90-A78B-0E808F295D41}">
   <ds:schemaRefs>
@@ -5248,6 +5427,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E32AD742-8CF8-4A25-BDB4-C877FB6C5FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5265,21 +5461,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF9DA147-3E0D-4271-B952-554C91C09EC2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56BF8649-3B4B-4285-B7D7-B1E422EBA2C5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
clarified date time format
clarified date time format
</commit_message>
<xml_diff>
--- a/excel/PTV Flows HDA analysis excel tool.xlsx
+++ b/excel/PTV Flows HDA analysis excel tool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luca.paone\github\PTV-Flows-tutorials\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAB72E2-4BCD-4539-B0DD-61B8C3B7C266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C12EE32F-0685-46D6-8D59-971475DD46EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
   <si>
     <t>your apiKey &gt;</t>
   </si>
@@ -263,9 +263,6 @@
     <t>toTime (ISO 8601 format) UTC</t>
   </si>
   <si>
-    <t>input date/time in your timezone accordingly with cell D5</t>
-  </si>
-  <si>
     <t>Hour Difference with UTC  (0,+1,+2,-1,-2  etc)</t>
   </si>
   <si>
@@ -338,7 +335,13 @@
     <t>For the "Get HDA KPI DETAILED data" button, the time interval between From and To must not exceed 24 hours.</t>
   </si>
   <si>
-    <t>yyyy-mm-dd UTC Time</t>
+    <t>input date/time in your timezone accordingly with cell D5, format is yyyy-mm-dd</t>
+  </si>
+  <si>
+    <t>hour format is hh:mm</t>
+  </si>
+  <si>
+    <t>yyyy-mm-dd hh:mm UTC Time</t>
   </si>
 </sst>
 </file>
@@ -672,9 +675,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -702,6 +702,10 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -3632,13 +3636,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
@@ -3688,9 +3692,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B4" s="13">
         <v>45717</v>
@@ -3699,7 +3703,7 @@
         <v>45717</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -3709,6 +3713,9 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
       <c r="B5" s="14">
         <v>0</v>
       </c>
@@ -3729,16 +3736,16 @@
       <c r="A6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="31">
         <f>IF($D$5&gt;0,B4+B5-TIME($D$5,0,0),B4+B5+TIME(-1*$D$5,0,0))</f>
         <v>45716.916666666664</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="31">
         <f>IF($D$5&gt;0,C4+C5-TIME($D$5,0,0),C4+C5+TIME(-1*$D$5,0,0))</f>
         <v>45717.915972222218</v>
       </c>
-      <c r="D6" s="25" t="s">
-        <v>51</v>
+      <c r="D6" s="34" t="s">
+        <v>52</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -3749,8 +3756,8 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="34"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
@@ -3789,7 +3796,7 @@
       <c r="E11" s="12"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
-      <c r="I11" s="33"/>
+      <c r="I11" s="32"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
@@ -3841,20 +3848,20 @@
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="30"/>
-      <c r="G17" s="31"/>
+      <c r="E17" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="29"/>
+      <c r="G17" s="30"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
@@ -5034,12 +5041,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -5069,12 +5076,12 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
@@ -5083,8 +5090,8 @@
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="26" t="s">
-        <v>50</v>
+      <c r="A15" s="25" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -5132,7 +5139,7 @@
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -5142,7 +5149,7 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>